<commit_message>
Resultados estables con 20 nodos antes de reemplazo MIP
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -965,35 +965,35 @@
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>[1, 13, 17, 16, 12, 1]</t>
+          <t>[1, 15, 11, 13, 17, 1]</t>
         </is>
       </c>
       <c r="AM3" t="n">
-        <v>4217</v>
+        <v>4354</v>
       </c>
       <c r="AN3" t="n">
-        <v>71.12444971666353</v>
+        <v>75.09009377717234</v>
       </c>
       <c r="AO3" t="b">
         <v>1</v>
       </c>
       <c r="AP3" t="n">
-        <v>-3.248755039127342</v>
+        <v>0</v>
       </c>
       <c r="AQ3" t="n">
-        <v>-3.248755039127342</v>
+        <v>0</v>
       </c>
       <c r="AR3" t="n">
-        <v>42.18638842779227</v>
+        <v>44.00551217271475</v>
       </c>
       <c r="AS3" t="n">
-        <v>-3.248755039127342</v>
+        <v>0</v>
       </c>
       <c r="AT3" t="n">
-        <v>2.157932179274366</v>
+        <v>5.236564079007809</v>
       </c>
       <c r="AU3" t="n">
-        <v>7.493478776381314</v>
+        <v>10.4042259990813</v>
       </c>
     </row>
     <row r="4">
@@ -1295,35 +1295,35 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>[3, 14, 4, 3]</t>
+          <t>[3, 4, 14, 3]</t>
         </is>
       </c>
       <c r="AM5" t="n">
-        <v>1730</v>
+        <v>1550</v>
       </c>
       <c r="AN5" t="n">
-        <v>63.30871336570848</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="AO5" t="b">
         <v>1</v>
       </c>
       <c r="AP5" t="n">
-        <v>0</v>
+        <v>-11.61290322580645</v>
       </c>
       <c r="AQ5" t="n">
-        <v>0</v>
+        <v>-11.61290322580645</v>
       </c>
       <c r="AR5" t="n">
-        <v>35.83815028901734</v>
+        <v>28.38709677419355</v>
       </c>
       <c r="AS5" t="n">
-        <v>0</v>
+        <v>-11.61290322580645</v>
       </c>
       <c r="AT5" t="n">
-        <v>0</v>
+        <v>-11.61290322580645</v>
       </c>
       <c r="AU5" t="n">
-        <v>0</v>
+        <v>-11.61290322580645</v>
       </c>
     </row>
     <row r="6">
@@ -1955,35 +1955,35 @@
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>[7, 6, 11, 13, 7]</t>
+          <t>[7, 15, 11, 6, 7]</t>
         </is>
       </c>
       <c r="AM9" t="n">
-        <v>3195</v>
+        <v>2583</v>
       </c>
       <c r="AN9" t="n">
-        <v>65.89413159769893</v>
+        <v>72.2774858316217</v>
       </c>
       <c r="AO9" t="b">
         <v>1</v>
       </c>
       <c r="AP9" t="n">
-        <v>28.29420970266041</v>
+        <v>11.30468447541618</v>
       </c>
       <c r="AQ9" t="n">
-        <v>15.68075117370892</v>
+        <v>-4.29732868757259</v>
       </c>
       <c r="AR9" t="n">
-        <v>98.27856025039124</v>
+        <v>97.87069299264421</v>
       </c>
       <c r="AS9" t="n">
-        <v>0</v>
+        <v>-23.69337979094077</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>-23.69337979094077</v>
       </c>
       <c r="AU9" t="n">
-        <v>10.82942097026604</v>
+        <v>-10.29810298102981</v>
       </c>
     </row>
     <row r="10">
@@ -2120,35 +2120,35 @@
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>[8, 11, 13, 1, 17, 8]</t>
+          <t>[8, 2, 18, 17, 1, 13, 8]</t>
         </is>
       </c>
       <c r="AM10" t="n">
-        <v>3966</v>
+        <v>3792</v>
       </c>
       <c r="AN10" t="n">
-        <v>76.8562911536078</v>
+        <v>76.75141659465383</v>
       </c>
       <c r="AO10" t="b">
         <v>1</v>
       </c>
       <c r="AP10" t="n">
-        <v>10.89258698940998</v>
+        <v>6.80379746835443</v>
       </c>
       <c r="AQ10" t="n">
-        <v>10.89258698940998</v>
+        <v>6.80379746835443</v>
       </c>
       <c r="AR10" t="n">
-        <v>30.98840141200202</v>
+        <v>27.82172995780591</v>
       </c>
       <c r="AS10" t="n">
-        <v>10.89258698940998</v>
+        <v>6.80379746835443</v>
       </c>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>-4.588607594936709</v>
       </c>
       <c r="AU10" t="n">
-        <v>0</v>
+        <v>-4.588607594936709</v>
       </c>
     </row>
     <row r="11">
@@ -2285,35 +2285,35 @@
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>[9, 19, 9]</t>
+          <t>[9, 2, 9]</t>
         </is>
       </c>
       <c r="AM11" t="n">
-        <v>-1961</v>
+        <v>-4042</v>
       </c>
       <c r="AN11" t="n">
-        <v>31.18836819706772</v>
+        <v>64.70237352474922</v>
       </c>
       <c r="AO11" t="b">
         <v>1</v>
       </c>
       <c r="AP11" t="n">
-        <v>-1.478837327893932</v>
+        <v>-52.20188025729837</v>
       </c>
       <c r="AQ11" t="n">
-        <v>-1.478837327893932</v>
+        <v>-52.20188025729837</v>
       </c>
       <c r="AR11" t="n">
-        <v>57.87863335033146</v>
+        <v>-23.40425531914894</v>
       </c>
       <c r="AS11" t="n">
-        <v>-1.478837327893932</v>
+        <v>-52.20188025729837</v>
       </c>
       <c r="AT11" t="n">
-        <v>-1.478837327893932</v>
+        <v>-52.20188025729837</v>
       </c>
       <c r="AU11" t="n">
-        <v>-1.478837327893932</v>
+        <v>-52.20188025729837</v>
       </c>
     </row>
     <row r="12">
@@ -3605,35 +3605,35 @@
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>[17, 11, 13, 1, 12, 17]</t>
+          <t>[17, 16, 12, 1, 13, 17]</t>
         </is>
       </c>
       <c r="AM19" t="n">
-        <v>3991</v>
+        <v>3963</v>
       </c>
       <c r="AN19" t="n">
-        <v>70.51893234490386</v>
+        <v>71.12444971666355</v>
       </c>
       <c r="AO19" t="b">
         <v>1</v>
       </c>
       <c r="AP19" t="n">
-        <v>2.179904785767978</v>
+        <v>1.488771132980066</v>
       </c>
       <c r="AQ19" t="n">
-        <v>2.179904785767978</v>
+        <v>1.488771132980066</v>
       </c>
       <c r="AR19" t="n">
-        <v>30.29315960912052</v>
+        <v>29.80065606863487</v>
       </c>
       <c r="AS19" t="n">
-        <v>0.7015785517414181</v>
+        <v>0</v>
       </c>
       <c r="AT19" t="n">
-        <v>0.7015785517414181</v>
+        <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>14.70809320972187</v>
+        <v>14.10547564976028</v>
       </c>
     </row>
     <row r="20">
@@ -3770,35 +3770,35 @@
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>[18, 2, 17, 13, 8, 18]</t>
+          <t>[18, 2, 17, 1, 13, 18]</t>
         </is>
       </c>
       <c r="AM20" t="n">
-        <v>4385</v>
+        <v>3921</v>
       </c>
       <c r="AN20" t="n">
-        <v>67.12246371278081</v>
+        <v>74.08000733194871</v>
       </c>
       <c r="AO20" t="b">
         <v>1</v>
       </c>
       <c r="AP20" t="n">
-        <v>23.60319270239453</v>
+        <v>14.56261157867891</v>
       </c>
       <c r="AQ20" t="n">
-        <v>23.60319270239453</v>
+        <v>14.56261157867891</v>
       </c>
       <c r="AR20" t="n">
-        <v>33.40935005701255</v>
+        <v>25.52920173425147</v>
       </c>
       <c r="AS20" t="n">
-        <v>14.8460661345496</v>
+        <v>4.769191532772251</v>
       </c>
       <c r="AT20" t="n">
-        <v>0</v>
+        <v>-11.83371588880388</v>
       </c>
       <c r="AU20" t="n">
-        <v>0</v>
+        <v>-11.83371588880388</v>
       </c>
     </row>
     <row r="21">
@@ -3935,35 +3935,35 @@
       </c>
       <c r="AL21" t="inlineStr">
         <is>
-          <t>[19, 2, 18, 19]</t>
+          <t>[19, 5, 14, 19]</t>
         </is>
       </c>
       <c r="AM21" t="n">
-        <v>2767</v>
+        <v>2223</v>
       </c>
       <c r="AN21" t="n">
-        <v>63.91144733431781</v>
+        <v>75.84533600861731</v>
       </c>
       <c r="AO21" t="b">
         <v>1</v>
       </c>
       <c r="AP21" t="n">
-        <v>19.66028189374774</v>
+        <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>19.66028189374774</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>7.914709071196241</v>
+        <v>-14.61988304093567</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>-24.47143499775079</v>
       </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>-24.47143499775079</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>-24.47143499775079</v>
       </c>
     </row>
   </sheetData>
@@ -4147,7 +4147,7 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>3382.05</v>
+        <v>3184.75</v>
       </c>
       <c r="D2" t="n">
         <v>2943.05</v>
@@ -4174,61 +4174,61 @@
         <v>-8.833356243192341</v>
       </c>
       <c r="L2" t="n">
-        <v>7790.83679485321</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>373.1798529624939</v>
+        <v>404.6290159225464</v>
       </c>
       <c r="N2" t="n">
-        <v>7409.356439113617</v>
+        <v>7649.89470243454</v>
       </c>
       <c r="O2" t="n">
-        <v>1.482546329498291</v>
+        <v>1.536357402801514</v>
       </c>
       <c r="P2" t="n">
-        <v>8387.486028671265</v>
+        <v>8317.92471408844</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.49001260146322</v>
+        <v>5.862709743029631</v>
       </c>
       <c r="R2" t="n">
         <v>40.01390176088972</v>
       </c>
       <c r="S2" t="n">
-        <v>0.7898274982858106</v>
+        <v>-5.43747405569674</v>
       </c>
       <c r="T2" t="n">
         <v>10.9676007005254</v>
       </c>
       <c r="U2" t="n">
-        <v>48.16472083394029</v>
+        <v>42.09489077760513</v>
       </c>
       <c r="V2" t="n">
         <v>193.9649122807018</v>
       </c>
       <c r="W2" t="n">
-        <v>2.435817910112684</v>
+        <v>-3.670144518854786</v>
       </c>
       <c r="X2" t="n">
-        <v>14.8460661345496</v>
+        <v>13.6098981077147</v>
       </c>
       <c r="Y2" t="n">
-        <v>2.080726623535156</v>
+        <v>2.080702781677246</v>
       </c>
       <c r="Z2" t="n">
-        <v>5.00723123550415</v>
+        <v>4.96666431427002</v>
       </c>
       <c r="AA2" t="n">
         <v>3096.4</v>
       </c>
       <c r="AB2" t="n">
-        <v>9.550321525471457</v>
+        <v>3.447866579208471</v>
       </c>
       <c r="AC2" t="n">
         <v>82.66666666666667</v>
       </c>
       <c r="AD2" t="n">
-        <v>197.3885655403137</v>
+        <v>193.420672416687</v>
       </c>
       <c r="AE2" t="n">
         <v>17.61153057898312</v>

</xml_diff>

<commit_message>
Nueva implementación MIP pero da timeout con 20 nodos
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ21"/>
+  <dimension ref="A1:AO21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -610,6 +610,31 @@
           <t>HGA-LNS Valid</t>
         </is>
       </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Status</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Route</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Reward</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Duration</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Valid</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -738,6 +763,25 @@
       <c r="AJ2" t="b">
         <v>1</v>
       </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>[0, 11, 13, 15, 0]</t>
+        </is>
+      </c>
+      <c r="AM2" t="n">
+        <v>3074</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>76.91766635133968</v>
+      </c>
+      <c r="AO2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -865,6 +909,29 @@
       </c>
       <c r="AJ3" t="b">
         <v>1</v>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>[1, 13, 12, 1]</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -994,6 +1061,29 @@
       <c r="AJ4" t="b">
         <v>1</v>
       </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>[2, 9, 2]</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1122,6 +1212,25 @@
       <c r="AJ5" t="b">
         <v>1</v>
       </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>[3, 14, 4, 3]</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>1730</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>63.30871336570848</v>
+      </c>
+      <c r="AO5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1250,6 +1359,25 @@
       <c r="AJ6" t="b">
         <v>1</v>
       </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>[4, 14, 3, 4]</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>1912</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>63.4815652406223</v>
+      </c>
+      <c r="AO6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1378,6 +1506,25 @@
       <c r="AJ7" t="b">
         <v>1</v>
       </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>[5, 4, 14, 5]</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>2617</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>72.10731512057799</v>
+      </c>
+      <c r="AO7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1506,6 +1653,29 @@
       <c r="AJ8" t="b">
         <v>1</v>
       </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>[6, 11, 13, 1, 15, 6]</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1634,6 +1804,25 @@
       <c r="AJ9" t="b">
         <v>1</v>
       </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>[7, 6, 11, 13, 7]</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>3195</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>65.89413159769893</v>
+      </c>
+      <c r="AO9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1762,6 +1951,29 @@
       <c r="AJ10" t="b">
         <v>1</v>
       </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>[8, 13, 8]</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1890,6 +2102,25 @@
       <c r="AJ11" t="b">
         <v>1</v>
       </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>[9, 14, 19, 9]</t>
+        </is>
+      </c>
+      <c r="AM11" t="n">
+        <v>-1932</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>60.31740986873555</v>
+      </c>
+      <c r="AO11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2018,6 +2249,25 @@
       <c r="AJ12" t="b">
         <v>1</v>
       </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>[10, 4, 14, 10]</t>
+        </is>
+      </c>
+      <c r="AM12" t="n">
+        <v>1425</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>64.55122978877812</v>
+      </c>
+      <c r="AO12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2146,6 +2396,29 @@
       <c r="AJ13" t="b">
         <v>1</v>
       </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>BoundaryMismatch</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>[11, 13, 1, 15, 6, 11]</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2274,6 +2547,25 @@
       <c r="AJ14" t="b">
         <v>1</v>
       </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>Infeasible</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2402,6 +2694,29 @@
       <c r="AJ15" t="b">
         <v>1</v>
       </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>[13, 7, 11, 13]</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO15" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2530,6 +2845,25 @@
       <c r="AJ16" t="b">
         <v>1</v>
       </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>[14, 19, 4, 14]</t>
+        </is>
+      </c>
+      <c r="AM16" t="n">
+        <v>5846</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>61.9406740584577</v>
+      </c>
+      <c r="AO16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2658,6 +2992,29 @@
       <c r="AJ17" t="b">
         <v>1</v>
       </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>[15, 6, 11, 13, 1, 15]</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO17" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2786,6 +3143,29 @@
       <c r="AJ18" t="b">
         <v>1</v>
       </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>[16, 12, 16]</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO18" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2914,6 +3294,25 @@
       <c r="AJ19" t="b">
         <v>1</v>
       </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>Infeasible</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3042,6 +3441,29 @@
       <c r="AJ20" t="b">
         <v>1</v>
       </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>TimeLimit</t>
+        </is>
+      </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>[18, 2, 17, 13, 8, 18]</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="AO20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3168,6 +3590,25 @@
         <v>63.91144733431781</v>
       </c>
       <c r="AJ21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>[19, 2, 18, 19]</t>
+        </is>
+      </c>
+      <c r="AM21" t="n">
+        <v>2767</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>63.91144733431781</v>
+      </c>
+      <c r="AO21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3182,7 +3623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3198,85 +3639,145 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>MIP Avg Reward</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Optimal Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Avg Inference (ms)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Avg Reward</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>DRL Real Avg Reward</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Reward</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HGA-LNS Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>HGA-LNS Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Reward</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Reward</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Avg Reward</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Reward</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>DRL Training Time (s)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MC-Rollout Avg Reward</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>MC-Rollout Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs MC-Rollout (%)</t>
         </is>
@@ -3292,54 +3793,90 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
+        <v>2292.666666666667</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>263581.7496418953</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3025.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>9.176992107739258</v>
+      </c>
+      <c r="H2" t="n">
+        <v>28.29420970266041</v>
+      </c>
+      <c r="I2" t="n">
         <v>2943.05</v>
       </c>
-      <c r="D2" t="n">
+      <c r="J2" t="n">
         <v>3347.2</v>
       </c>
-      <c r="E2" t="n">
+      <c r="K2" t="n">
+        <v>0.3831417624521072</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3.448275862068965</v>
+      </c>
+      <c r="M2" t="n">
         <v>1773.2</v>
       </c>
-      <c r="F2" t="n">
+      <c r="N2" t="n">
+        <v>62.66021437385476</v>
+      </c>
+      <c r="O2" t="n">
+        <v>193.9649122807018</v>
+      </c>
+      <c r="P2" t="n">
         <v>3276.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>1885</v>
       </c>
-      <c r="H2" t="n">
+      <c r="T2" t="n">
         <v>3252.85</v>
       </c>
-      <c r="I2" t="n">
+      <c r="U2" t="n">
         <v>59.66731517363043</v>
       </c>
-      <c r="J2" t="n">
+      <c r="V2" t="n">
         <v>-8.833356243192341</v>
       </c>
-      <c r="K2" t="n">
+      <c r="W2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="n">
-        <v>383.0421924591064</v>
-      </c>
-      <c r="M2" t="n">
-        <v>7881.504905223846</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1.450932025909424</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2.054500579833984</v>
-      </c>
-      <c r="P2" t="n">
-        <v>4.84316349029541</v>
-      </c>
-      <c r="Q2" t="n">
+      <c r="X2" t="n">
+        <v>414.389705657959</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>7619.054198265076</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1.448440551757812</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2.086806297302246</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>4.744076728820801</v>
+      </c>
+      <c r="AC2" t="n">
         <v>3096.4</v>
       </c>
-      <c r="R2" t="n">
-        <v>196.2643027305603</v>
-      </c>
-      <c r="S2" t="n">
+      <c r="AD2" t="n">
+        <v>195.4564213752747</v>
+      </c>
+      <c r="AE2" t="n">
         <v>17.61153057898312</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Primera prueba al agregar DP
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -612,27 +612,27 @@
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>MIP Status</t>
+          <t>LS-Exact Status</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>MIP Route</t>
+          <t>LS-Exact Route</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>MIP Reward</t>
+          <t>LS-Exact Reward</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>MIP Duration</t>
+          <t>LS-Exact Duration</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>MIP Valid</t>
+          <t>LS-Exact Valid</t>
         </is>
       </c>
     </row>
@@ -912,26 +912,22 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>[1, 13, 12, 1]</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>[1, 15, 11, 13, 17, 1]</t>
+        </is>
+      </c>
+      <c r="AM3" t="n">
+        <v>4354</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>75.09009377717234</v>
       </c>
       <c r="AO3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1063,26 +1059,22 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>[2, 9, 2]</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>[2, 18, 11, 13, 8, 2]</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>4063</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>68.56140072641273</v>
       </c>
       <c r="AO4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1655,7 +1647,7 @@
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
@@ -1663,18 +1655,14 @@
           <t>[6, 11, 13, 1, 15, 6]</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN8" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="AM8" t="n">
+        <v>4122</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>76.13400093175433</v>
       </c>
       <c r="AO8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1953,26 +1941,22 @@
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>[8, 13, 8]</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>[8, 11, 13, 1, 17, 8]</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>3966</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>76.8562911536078</v>
       </c>
       <c r="AO10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2398,7 +2382,7 @@
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>BoundaryMismatch</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
@@ -2406,18 +2390,14 @@
           <t>[11, 13, 1, 15, 6, 11]</t>
         </is>
       </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="AM13" t="n">
+        <v>4568</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>76.13400093175433</v>
       </c>
       <c r="AO13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2549,22 +2529,22 @@
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>Infeasible</t>
-        </is>
-      </c>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>[12, 1, 13, 17, 16, 12]</t>
+        </is>
+      </c>
+      <c r="AM14" t="n">
+        <v>4631</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>71.12444971666355</v>
       </c>
       <c r="AO14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2696,26 +2676,22 @@
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>[13, 7, 11, 13]</t>
-        </is>
-      </c>
-      <c r="AM15" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>[13, 17, 1, 15, 11, 13]</t>
+        </is>
+      </c>
+      <c r="AM15" t="n">
+        <v>5017</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>75.09009377717236</v>
       </c>
       <c r="AO15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2994,7 +2970,7 @@
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
@@ -3002,18 +2978,14 @@
           <t>[15, 6, 11, 13, 1, 15]</t>
         </is>
       </c>
-      <c r="AM17" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="AM17" t="n">
+        <v>4316</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>76.13400093175433</v>
       </c>
       <c r="AO17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -3145,26 +3117,22 @@
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>[16, 12, 16]</t>
-        </is>
-      </c>
-      <c r="AM18" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN18" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>[16, 12, 1, 13, 17, 16]</t>
+        </is>
+      </c>
+      <c r="AM18" t="n">
+        <v>3760</v>
+      </c>
+      <c r="AN18" t="n">
+        <v>71.12444971666353</v>
       </c>
       <c r="AO18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -3296,22 +3264,22 @@
       </c>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>Infeasible</t>
-        </is>
-      </c>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN19" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>[17, 11, 13, 1, 12, 17]</t>
+        </is>
+      </c>
+      <c r="AM19" t="n">
+        <v>3991</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>70.51893234490386</v>
       </c>
       <c r="AO19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -3443,7 +3411,7 @@
       </c>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>TimeLimit</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="AL20" t="inlineStr">
@@ -3451,18 +3419,14 @@
           <t>[18, 2, 17, 13, 8, 18]</t>
         </is>
       </c>
-      <c r="AM20" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="AN20" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="AM20" t="n">
+        <v>4385</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>67.12246371278081</v>
       </c>
       <c r="AO20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -3623,7 +3587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3639,145 +3603,105 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>MIP Avg Reward</t>
+          <t>LS-Exact Avg Reward</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>MIP Optimal Count</t>
+          <t>DRL Det Avg Reward</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>MIP Avg Inference (ms)</t>
+          <t>DRL Det Gap vs LS-Exact (%)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>DRL Det Avg Reward</t>
+          <t>DRL Real Avg Reward</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>DRL Det Gap vs MIP Avg (%)</t>
+          <t>HGA-LNS Avg Reward</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>DRL Det Gap vs MIP Max (%)</t>
+          <t>RH-Greedy Avg Reward</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Avg Reward</t>
+          <t>RH-Lookahead Avg Reward</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Avg Reward</t>
+          <t>RH-Greedy Real Avg Reward</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Gap vs MIP Avg (%)</t>
+          <t>RH-Lookahead Real Avg Reward</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Gap vs MIP Max (%)</t>
+          <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Avg Reward</t>
+          <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Gap vs MIP Avg (%)</t>
+          <t>DRL Training Time (s)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Gap vs MIP Max (%)</t>
+          <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>RH-Lookahead Avg Reward</t>
+          <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>RH-Lookahead Gap vs MIP Avg (%)</t>
+          <t>LS-Exact Avg Inference (ms)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>RH-Lookahead Gap vs MIP Max (%)</t>
+          <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Real Avg Reward</t>
+          <t>RH-Lookahead Avg Inference (ms)</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>RH-Lookahead Real Avg Reward</t>
+          <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
+          <t>MC-Rollout Avg Reward</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
+          <t>MC-Rollout Avg Inference (ms)</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Training Time (s)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Real Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>HGA-LNS Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Greedy Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Lookahead Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Lookahead Real Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>MC-Rollout Avg Reward</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>MC-Rollout Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs MC-Rollout (%)</t>
         </is>
@@ -3793,90 +3717,66 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>2292.666666666667</v>
+        <v>3390.35</v>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>3025.6</v>
       </c>
       <c r="E2" t="n">
-        <v>263581.7496418953</v>
+        <v>9.811402187028291</v>
       </c>
       <c r="F2" t="n">
-        <v>3025.6</v>
+        <v>2943.05</v>
       </c>
       <c r="G2" t="n">
-        <v>9.176992107739258</v>
+        <v>3347.2</v>
       </c>
       <c r="H2" t="n">
-        <v>28.29420970266041</v>
+        <v>1773.2</v>
       </c>
       <c r="I2" t="n">
-        <v>2943.05</v>
+        <v>3276.7</v>
       </c>
       <c r="J2" t="n">
-        <v>3347.2</v>
+        <v>1885</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3831417624521072</v>
+        <v>3252.85</v>
       </c>
       <c r="L2" t="n">
-        <v>3.448275862068965</v>
+        <v>59.66731517363043</v>
       </c>
       <c r="M2" t="n">
-        <v>1773.2</v>
+        <v>-8.833356243192341</v>
       </c>
       <c r="N2" t="n">
-        <v>62.66021437385476</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>193.9649122807018</v>
+        <v>383.8558077812195</v>
       </c>
       <c r="P2" t="n">
-        <v>3276.7</v>
+        <v>7432.907068729401</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>2.972865104675293</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>1.415610313415527</v>
       </c>
       <c r="S2" t="n">
-        <v>1885</v>
+        <v>2.034866809844971</v>
       </c>
       <c r="T2" t="n">
-        <v>3252.85</v>
+        <v>4.810333251953125</v>
       </c>
       <c r="U2" t="n">
-        <v>59.66731517363043</v>
+        <v>3096.4</v>
       </c>
       <c r="V2" t="n">
-        <v>-8.833356243192341</v>
+        <v>194.4154024124146</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>414.389705657959</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>7619.054198265076</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>1.448440551757812</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>2.086806297302246</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>4.744076728820801</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>3096.4</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>195.4564213752747</v>
-      </c>
-      <c r="AE2" t="n">
         <v>17.61153057898312</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Primera prueba al agregar Label setting estocastico
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO21"/>
+  <dimension ref="A1:AT21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -635,6 +635,31 @@
           <t>LS-Exact Valid</t>
         </is>
       </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Status</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Route</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Reward</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Duration</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Valid</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -782,6 +807,25 @@
       <c r="AO2" t="b">
         <v>1</v>
       </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>[0, 11, 13, 15, 0]</t>
+        </is>
+      </c>
+      <c r="AR2" t="n">
+        <v>3074</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>76.91766635133968</v>
+      </c>
+      <c r="AT2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -927,6 +971,25 @@
         <v>75.09009377717234</v>
       </c>
       <c r="AO3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>[1, 15, 11, 13, 17, 1]</t>
+        </is>
+      </c>
+      <c r="AR3" t="n">
+        <v>4354</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>75.09009377717234</v>
+      </c>
+      <c r="AT3" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1076,6 +1139,25 @@
       <c r="AO4" t="b">
         <v>1</v>
       </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>[2, 8, 13, 1, 17, 18, 2]</t>
+        </is>
+      </c>
+      <c r="AR4" t="n">
+        <v>3913</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>76.92379758974533</v>
+      </c>
+      <c r="AT4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1223,6 +1305,25 @@
       <c r="AO5" t="b">
         <v>1</v>
       </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>[3, 14, 4, 3]</t>
+        </is>
+      </c>
+      <c r="AR5" t="n">
+        <v>1730</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>63.30871336570848</v>
+      </c>
+      <c r="AT5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1370,6 +1471,25 @@
       <c r="AO6" t="b">
         <v>1</v>
       </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>[4, 14, 3, 4]</t>
+        </is>
+      </c>
+      <c r="AR6" t="n">
+        <v>1912</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>63.4815652406223</v>
+      </c>
+      <c r="AT6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1517,6 +1637,25 @@
       <c r="AO7" t="b">
         <v>1</v>
       </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>[5, 4, 14, 5]</t>
+        </is>
+      </c>
+      <c r="AR7" t="n">
+        <v>2617</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>72.10731512057799</v>
+      </c>
+      <c r="AT7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1664,6 +1803,25 @@
       <c r="AO8" t="b">
         <v>1</v>
       </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>[6, 11, 13, 1, 15, 6]</t>
+        </is>
+      </c>
+      <c r="AR8" t="n">
+        <v>4122</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>76.13400093175433</v>
+      </c>
+      <c r="AT8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1811,6 +1969,25 @@
       <c r="AO9" t="b">
         <v>1</v>
       </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>[7, 6, 11, 13, 7]</t>
+        </is>
+      </c>
+      <c r="AR9" t="n">
+        <v>3195</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>65.89413159769893</v>
+      </c>
+      <c r="AT9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1958,6 +2135,25 @@
       <c r="AO10" t="b">
         <v>1</v>
       </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>[8, 11, 13, 1, 17, 8]</t>
+        </is>
+      </c>
+      <c r="AR10" t="n">
+        <v>3966</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>76.8562911536078</v>
+      </c>
+      <c r="AT10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2105,6 +2301,25 @@
       <c r="AO11" t="b">
         <v>1</v>
       </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>[9, 14, 19, 9]</t>
+        </is>
+      </c>
+      <c r="AR11" t="n">
+        <v>-1932</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>60.31740986873555</v>
+      </c>
+      <c r="AT11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2252,6 +2467,25 @@
       <c r="AO12" t="b">
         <v>1</v>
       </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>[10, 4, 14, 10]</t>
+        </is>
+      </c>
+      <c r="AR12" t="n">
+        <v>1425</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>64.55122978877812</v>
+      </c>
+      <c r="AT12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2399,6 +2633,25 @@
       <c r="AO13" t="b">
         <v>1</v>
       </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>[11, 13, 1, 15, 6, 11]</t>
+        </is>
+      </c>
+      <c r="AR13" t="n">
+        <v>4568</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>76.13400093175433</v>
+      </c>
+      <c r="AT13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2546,6 +2799,25 @@
       <c r="AO14" t="b">
         <v>1</v>
       </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>[12, 1, 13, 17, 16, 12]</t>
+        </is>
+      </c>
+      <c r="AR14" t="n">
+        <v>4631</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>71.12444971666355</v>
+      </c>
+      <c r="AT14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2693,6 +2965,25 @@
       <c r="AO15" t="b">
         <v>1</v>
       </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>[13, 17, 1, 15, 11, 13]</t>
+        </is>
+      </c>
+      <c r="AR15" t="n">
+        <v>5017</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>75.09009377717236</v>
+      </c>
+      <c r="AT15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2840,6 +3131,25 @@
       <c r="AO16" t="b">
         <v>1</v>
       </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>[14, 19, 4, 14]</t>
+        </is>
+      </c>
+      <c r="AR16" t="n">
+        <v>5846</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>61.9406740584577</v>
+      </c>
+      <c r="AT16" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2987,6 +3297,25 @@
       <c r="AO17" t="b">
         <v>1</v>
       </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>[15, 6, 11, 13, 1, 15]</t>
+        </is>
+      </c>
+      <c r="AR17" t="n">
+        <v>4316</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>76.13400093175433</v>
+      </c>
+      <c r="AT17" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -3134,6 +3463,25 @@
       <c r="AO18" t="b">
         <v>1</v>
       </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>[16, 12, 1, 13, 17, 16]</t>
+        </is>
+      </c>
+      <c r="AR18" t="n">
+        <v>3760</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>71.12444971666353</v>
+      </c>
+      <c r="AT18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3281,6 +3629,25 @@
       <c r="AO19" t="b">
         <v>1</v>
       </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>[17, 11, 13, 1, 12, 17]</t>
+        </is>
+      </c>
+      <c r="AR19" t="n">
+        <v>3991</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>70.51893234490386</v>
+      </c>
+      <c r="AT19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3428,6 +3795,25 @@
       <c r="AO20" t="b">
         <v>1</v>
       </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>[18, 2, 17, 13, 8, 18]</t>
+        </is>
+      </c>
+      <c r="AR20" t="n">
+        <v>4385</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>67.12246371278081</v>
+      </c>
+      <c r="AT20" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3573,6 +3959,25 @@
         <v>63.91144733431781</v>
       </c>
       <c r="AO21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>[19, 2, 18, 19]</t>
+        </is>
+      </c>
+      <c r="AR21" t="n">
+        <v>2767</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>63.91144733431781</v>
+      </c>
+      <c r="AT21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3587,7 +3992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3623,85 +4028,100 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>LS-Oracle Avg Reward</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Gap vs LS-Oracle (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>LS-Oracle Avg Inference (ms)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>HGA-LNS Avg Reward</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Reward</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Reward</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Avg Reward</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Reward</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DRL Training Time (s)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>LS-Exact Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>MC-Rollout Avg Reward</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MC-Rollout Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs MC-Rollout (%)</t>
         </is>
@@ -3729,54 +4149,63 @@
         <v>2943.05</v>
       </c>
       <c r="G2" t="n">
+        <v>3382.85</v>
+      </c>
+      <c r="H2" t="n">
+        <v>11.55722551944427</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7.904839515686036</v>
+      </c>
+      <c r="J2" t="n">
         <v>3347.2</v>
       </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
         <v>1773.2</v>
       </c>
-      <c r="I2" t="n">
+      <c r="L2" t="n">
         <v>3276.7</v>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>1885</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N2" t="n">
         <v>3252.85</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O2" t="n">
         <v>59.66731517363043</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P2" t="n">
         <v>-8.833356243192341</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="n">
-        <v>383.8558077812195</v>
-      </c>
-      <c r="P2" t="n">
-        <v>7432.907068729401</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>2.972865104675293</v>
-      </c>
       <c r="R2" t="n">
-        <v>1.415610313415527</v>
+        <v>383.522367477417</v>
       </c>
       <c r="S2" t="n">
-        <v>2.034866809844971</v>
+        <v>7969.380605220795</v>
       </c>
       <c r="T2" t="n">
-        <v>4.810333251953125</v>
+        <v>3.004300594329834</v>
       </c>
       <c r="U2" t="n">
+        <v>1.411211490631104</v>
+      </c>
+      <c r="V2" t="n">
+        <v>2.011573314666748</v>
+      </c>
+      <c r="W2" t="n">
+        <v>4.694223403930664</v>
+      </c>
+      <c r="X2" t="n">
         <v>3096.4</v>
       </c>
-      <c r="V2" t="n">
-        <v>194.4154024124146</v>
-      </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
+        <v>190.9183025360107</v>
+      </c>
+      <c r="Z2" t="n">
         <v>17.61153057898312</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejora de GAP del DRL
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -673,28 +673,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[0, 1, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2297</v>
+        <v>2583</v>
       </c>
       <c r="F2" t="n">
-        <v>56.15262485093308</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[0, 1, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2297</v>
+        <v>2583</v>
       </c>
       <c r="J2" t="n">
-        <v>56.15262485093308</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="K2" t="b">
         <v>1</v>
@@ -1005,14 +1005,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[2, 18, 11, 13, 2]</t>
+          <t>[2, 11, 13, 8, 18, 2]</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3586</v>
+        <v>3794</v>
       </c>
       <c r="F4" t="n">
-        <v>63.95790717979659</v>
+        <v>71.86492405207225</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -1337,28 +1337,28 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[4, 5, 14, 4]</t>
+          <t>[4, 14, 3, 4]</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1733</v>
+        <v>1912</v>
       </c>
       <c r="F6" t="n">
-        <v>72.12551059405325</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[4, 5, 14, 4]</t>
+          <t>[4, 14, 3, 4]</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1733</v>
+        <v>1912</v>
       </c>
       <c r="J6" t="n">
-        <v>72.12551059405325</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="K6" t="b">
         <v>1</v>
@@ -1669,28 +1669,28 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>[6, 0, 15, 11, 6]</t>
+          <t>[6, 13, 1, 15, 6]</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2926</v>
+        <v>3561</v>
       </c>
       <c r="F8" t="n">
-        <v>64.88257727261286</v>
+        <v>75.87368123652222</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[6, 0, 15, 11, 6]</t>
+          <t>[6, 13, 1, 15, 6]</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2926</v>
+        <v>3561</v>
       </c>
       <c r="J8" t="n">
-        <v>64.88257727261286</v>
+        <v>75.87368123652222</v>
       </c>
       <c r="K8" t="b">
         <v>1</v>
@@ -1835,28 +1835,28 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>[7, 13, 11, 6, 7]</t>
+          <t>[7, 11, 13, 7]</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2694</v>
+        <v>2849</v>
       </c>
       <c r="F9" t="n">
-        <v>65.84630455243327</v>
+        <v>64.95063789465291</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[7, 8, 7]</t>
+          <t>[7, 11, 13, 7]</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2291</v>
+        <v>2849</v>
       </c>
       <c r="J9" t="n">
-        <v>72.81063071208843</v>
+        <v>64.95063789465291</v>
       </c>
       <c r="K9" t="b">
         <v>1</v>
@@ -3163,14 +3163,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[15, 6, 0, 15]</t>
+          <t>[15, 6, 7, 15]</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2589</v>
+        <v>3397</v>
       </c>
       <c r="F17" t="n">
-        <v>56.19291514611906</v>
+        <v>63.5878237051279</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -3329,14 +3329,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>[16, 12, 15, 1, 16]</t>
+          <t>[16, 12, 13, 1, 16]</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2900</v>
+        <v>3669</v>
       </c>
       <c r="F18" t="n">
-        <v>74.90639473783661</v>
+        <v>63.61202657160617</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
@@ -3661,28 +3661,28 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>[18, 1, 13, 2, 18]</t>
+          <t>[18, 17, 13, 8, 18]</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3350</v>
+        <v>3730</v>
       </c>
       <c r="F20" t="n">
-        <v>71.62834258031488</v>
+        <v>61.71021669731303</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>[18, 1, 13, 2, 18]</t>
+          <t>[18, 17, 13, 8, 18]</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>3350</v>
+        <v>3730</v>
       </c>
       <c r="J20" t="n">
-        <v>71.62834258031488</v>
+        <v>61.71021669731303</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -3827,28 +3827,28 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>[19, 5, 14, 19]</t>
+          <t>[19, 2, 18, 19]</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2223</v>
+        <v>2767</v>
       </c>
       <c r="F21" t="n">
-        <v>75.84533600861731</v>
+        <v>63.91144733431781</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>[19, 5, 14, 19]</t>
+          <t>[19, 2, 18, 19]</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2223</v>
+        <v>2767</v>
       </c>
       <c r="J21" t="n">
-        <v>75.84533600861731</v>
+        <v>63.91144733431781</v>
       </c>
       <c r="K21" t="b">
         <v>1</v>
@@ -4140,22 +4140,22 @@
         <v>3390.35</v>
       </c>
       <c r="D2" t="n">
-        <v>3025.6</v>
+        <v>3154.7</v>
       </c>
       <c r="E2" t="n">
-        <v>9.811402187028291</v>
+        <v>5.818308007384312</v>
       </c>
       <c r="F2" t="n">
-        <v>2943.05</v>
+        <v>3141.25</v>
       </c>
       <c r="G2" t="n">
         <v>3382.85</v>
       </c>
       <c r="H2" t="n">
-        <v>11.55722551944427</v>
+        <v>5.970365252464813</v>
       </c>
       <c r="I2" t="n">
-        <v>7.904839515686036</v>
+        <v>8.101248741149902</v>
       </c>
       <c r="J2" t="n">
         <v>3347.2</v>
@@ -4173,40 +4173,40 @@
         <v>3252.85</v>
       </c>
       <c r="O2" t="n">
-        <v>59.66731517363043</v>
+        <v>67.75256456918915</v>
       </c>
       <c r="P2" t="n">
-        <v>-8.833356243192341</v>
+        <v>-2.96438466774765</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>7812.454636096954</v>
       </c>
       <c r="R2" t="n">
-        <v>383.522367477417</v>
+        <v>652.4883508682251</v>
       </c>
       <c r="S2" t="n">
-        <v>7969.380605220795</v>
+        <v>7478.735256195068</v>
       </c>
       <c r="T2" t="n">
-        <v>3.004300594329834</v>
+        <v>3.070402145385742</v>
       </c>
       <c r="U2" t="n">
-        <v>1.411211490631104</v>
+        <v>1.513528823852539</v>
       </c>
       <c r="V2" t="n">
-        <v>2.011573314666748</v>
+        <v>2.263796329498291</v>
       </c>
       <c r="W2" t="n">
-        <v>4.694223403930664</v>
+        <v>5.157864093780518</v>
       </c>
       <c r="X2" t="n">
         <v>3096.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>190.9183025360107</v>
+        <v>203.4412503242493</v>
       </c>
       <c r="Z2" t="n">
-        <v>17.61153057898312</v>
+        <v>23.84719004078682</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados luego de eliminar n eval de 5
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -2679,14 +2679,14 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[12, 13, 1, 17, 12]</t>
+          <t>[12, 13, 17, 16, 12]</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>3615</v>
+        <v>4294</v>
       </c>
       <c r="J14" t="n">
-        <v>62.93765939747976</v>
+        <v>67.42434623698556</v>
       </c>
       <c r="K14" t="b">
         <v>1</v>
@@ -4140,10 +4140,10 @@
         <v>3390.35</v>
       </c>
       <c r="D2" t="n">
-        <v>3154.7</v>
+        <v>3188.65</v>
       </c>
       <c r="E2" t="n">
-        <v>5.818308007384312</v>
+        <v>5.085205005872759</v>
       </c>
       <c r="F2" t="n">
         <v>3141.25</v>
@@ -4155,7 +4155,7 @@
         <v>5.970365252464813</v>
       </c>
       <c r="I2" t="n">
-        <v>8.101248741149902</v>
+        <v>7.770872116088867</v>
       </c>
       <c r="J2" t="n">
         <v>3347.2</v>
@@ -4173,40 +4173,40 @@
         <v>3252.85</v>
       </c>
       <c r="O2" t="n">
-        <v>67.75256456918915</v>
+        <v>66.64456233421751</v>
       </c>
       <c r="P2" t="n">
-        <v>-2.96438466774765</v>
+        <v>-3.430837573205033</v>
       </c>
       <c r="Q2" t="n">
-        <v>7812.454636096954</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>652.4883508682251</v>
+        <v>150.0608444213867</v>
       </c>
       <c r="S2" t="n">
-        <v>7478.735256195068</v>
+        <v>7401.469838619232</v>
       </c>
       <c r="T2" t="n">
-        <v>3.070402145385742</v>
+        <v>2.950823307037354</v>
       </c>
       <c r="U2" t="n">
-        <v>1.513528823852539</v>
+        <v>1.392817497253418</v>
       </c>
       <c r="V2" t="n">
-        <v>2.263796329498291</v>
+        <v>2.011954784393311</v>
       </c>
       <c r="W2" t="n">
-        <v>5.157864093780518</v>
+        <v>4.62416410446167</v>
       </c>
       <c r="X2" t="n">
         <v>3096.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>203.4412503242493</v>
+        <v>189.0630125999451</v>
       </c>
       <c r="Z2" t="n">
-        <v>23.84719004078682</v>
+        <v>1.448456271799506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados luego de eliminar n eval de 30 en MC
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -4155,7 +4155,7 @@
         <v>5.970365252464813</v>
       </c>
       <c r="I2" t="n">
-        <v>7.770872116088867</v>
+        <v>7.698905467987061</v>
       </c>
       <c r="J2" t="n">
         <v>3347.2</v>
@@ -4182,28 +4182,28 @@
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>150.0608444213867</v>
+        <v>150.1246333122253</v>
       </c>
       <c r="S2" t="n">
-        <v>7401.469838619232</v>
+        <v>7576.946997642517</v>
       </c>
       <c r="T2" t="n">
-        <v>2.950823307037354</v>
+        <v>2.951574325561523</v>
       </c>
       <c r="U2" t="n">
-        <v>1.392817497253418</v>
+        <v>1.450872421264648</v>
       </c>
       <c r="V2" t="n">
-        <v>2.011954784393311</v>
+        <v>2.06836462020874</v>
       </c>
       <c r="W2" t="n">
-        <v>4.62416410446167</v>
+        <v>4.678583145141602</v>
       </c>
       <c r="X2" t="n">
         <v>3096.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>189.0630125999451</v>
+        <v>7.922196388244629</v>
       </c>
       <c r="Z2" t="n">
         <v>1.448456271799506</v>

</xml_diff>

<commit_message>
Gap estocastico del DRL de 1.6%
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -673,14 +673,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[0, 13, 1, 0]</t>
+          <t>[0, 11, 13, 15, 0]</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2583</v>
+        <v>3074</v>
       </c>
       <c r="F2" t="n">
-        <v>76.65434719173314</v>
+        <v>76.91766635133968</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -1835,14 +1835,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>[7, 11, 13, 7]</t>
+          <t>[7, 6, 11, 13, 7]</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2849</v>
+        <v>3195</v>
       </c>
       <c r="F9" t="n">
-        <v>64.95063789465291</v>
+        <v>65.89413159769893</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -2001,14 +2001,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[8, 15, 11, 13, 8]</t>
+          <t>[8, 11, 13, 1, 17, 8]</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3534</v>
+        <v>3966</v>
       </c>
       <c r="F10" t="n">
-        <v>72.90445852841761</v>
+        <v>76.8562911536078</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -2665,14 +2665,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>[12, 13, 1, 17, 12]</t>
+          <t>[12, 13, 17, 16, 12]</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3615</v>
+        <v>4294</v>
       </c>
       <c r="F14" t="n">
-        <v>62.93765939747976</v>
+        <v>67.42434623698556</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
@@ -2831,14 +2831,14 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>[13, 17, 16, 12, 1, 13]</t>
+          <t>[13, 17, 1, 15, 11, 13]</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>4902</v>
+        <v>5017</v>
       </c>
       <c r="F15" t="n">
-        <v>71.12444971666355</v>
+        <v>75.09009377717236</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
@@ -3163,14 +3163,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>[15, 6, 7, 15]</t>
+          <t>[15, 11, 13, 0, 15]</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3397</v>
+        <v>4052</v>
       </c>
       <c r="F17" t="n">
-        <v>63.5878237051279</v>
+        <v>74.50924346940734</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -3495,14 +3495,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>[17, 1, 15, 11, 13, 17]</t>
+          <t>[17, 11, 13, 1, 12, 17]</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3904</v>
+        <v>3991</v>
       </c>
       <c r="F19" t="n">
-        <v>75.09009377717236</v>
+        <v>70.51893234490386</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
@@ -3661,14 +3661,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>[18, 17, 13, 8, 18]</t>
+          <t>[18, 2, 17, 13, 8, 18]</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3730</v>
+        <v>4385</v>
       </c>
       <c r="F20" t="n">
-        <v>61.71021669731303</v>
+        <v>67.12246371278081</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
@@ -4146,16 +4146,16 @@
         <v>5.085205005872759</v>
       </c>
       <c r="F2" t="n">
-        <v>3141.25</v>
+        <v>3314.25</v>
       </c>
       <c r="G2" t="n">
         <v>3382.85</v>
       </c>
       <c r="H2" t="n">
-        <v>5.970365252464813</v>
+        <v>1.623253828057071</v>
       </c>
       <c r="I2" t="n">
-        <v>7.698905467987061</v>
+        <v>8.209049701690674</v>
       </c>
       <c r="J2" t="n">
         <v>3347.2</v>
@@ -4173,40 +4173,40 @@
         <v>3252.85</v>
       </c>
       <c r="O2" t="n">
-        <v>66.64456233421751</v>
+        <v>75.82228116710876</v>
       </c>
       <c r="P2" t="n">
-        <v>-3.430837573205033</v>
+        <v>1.887575510705999</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>150.1246333122253</v>
+        <v>224.4969129562378</v>
       </c>
       <c r="S2" t="n">
-        <v>7576.946997642517</v>
+        <v>7469.397020339966</v>
       </c>
       <c r="T2" t="n">
-        <v>2.951574325561523</v>
+        <v>3.013384342193604</v>
       </c>
       <c r="U2" t="n">
-        <v>1.450872421264648</v>
+        <v>1.457607746124268</v>
       </c>
       <c r="V2" t="n">
-        <v>2.06836462020874</v>
+        <v>2.092480659484863</v>
       </c>
       <c r="W2" t="n">
-        <v>4.678583145141602</v>
+        <v>4.923582077026367</v>
       </c>
       <c r="X2" t="n">
         <v>3096.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>7.922196388244629</v>
+        <v>8.022630214691162</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.448456271799506</v>
+        <v>7.035589717090812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados tras paralelizacion Nivel 1
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Per Node Results" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Stochastic Descriptive Stats" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wilcoxon Significance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PPO Convergence" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +46,27 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00548235"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +111,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -138,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +254,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -622,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2.96252171198527</v>
+        <v>2.099132537841797</v>
       </c>
     </row>
     <row r="4">
@@ -632,13 +734,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3321.083333333333</v>
+        <v>3314.616666666667</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>6.546824241565571</v>
+        <v>6.711958732542758</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>211.2622380256653</v>
+        <v>149.0353544553121</v>
       </c>
     </row>
     <row r="5">
@@ -648,13 +750,13 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>3554.733333333333</v>
+        <v>3585.483333333333</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.7176890945131639</v>
+        <v>0.05724222139238529</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>7445.640242099762</v>
+        <v>1740.631985664368</v>
       </c>
     </row>
     <row r="6">
@@ -670,7 +772,7 @@
         <v>4.612965002829824</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.039178212483724</v>
+        <v>1.154224077860514</v>
       </c>
     </row>
     <row r="7">
@@ -680,13 +782,13 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>2187.15</v>
+        <v>2300.75</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>41.75591774187075</v>
+        <v>39.86581939848013</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1.483329137166341</v>
+        <v>0.3040035565694173</v>
       </c>
     </row>
     <row r="9">
@@ -734,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>7.858033974965412</v>
+        <v>7.55076805750529</v>
       </c>
     </row>
     <row r="12">
@@ -750,7 +852,7 @@
         <v>1.940915761618184</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>211.2622380256653</v>
+        <v>149.0353544553121</v>
       </c>
     </row>
     <row r="13">
@@ -766,7 +868,7 @@
         <v>4.545012160007144</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>4.682616392771402</v>
+        <v>4.09390926361084</v>
       </c>
     </row>
     <row r="14">
@@ -776,10 +878,10 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2355.15</v>
+        <v>2404.716666666667</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>35.84623112449583</v>
+        <v>36.10069757805525</v>
       </c>
       <c r="D14" s="3" t="n"/>
     </row>
@@ -796,7 +898,7 @@
         <v>7.919557852777054</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>7.791761557261149</v>
+        <v>4.095109303792318</v>
       </c>
     </row>
     <row r="17">
@@ -826,7 +928,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0</v>
+        <v>13105.90102243423</v>
       </c>
     </row>
     <row r="20">
@@ -836,7 +938,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>211.2622380256653</v>
+        <v>149.0353544553121</v>
       </c>
     </row>
     <row r="21">
@@ -846,7 +948,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>7445.640242099762</v>
+        <v>1740.631985664368</v>
       </c>
     </row>
     <row r="22">
@@ -856,7 +958,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>2.96252171198527</v>
+        <v>2.099132537841797</v>
       </c>
     </row>
     <row r="23">
@@ -866,7 +968,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>1.483329137166341</v>
+        <v>0.3040035565694173</v>
       </c>
     </row>
     <row r="24">
@@ -876,7 +978,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>2.039178212483724</v>
+        <v>1.154224077860514</v>
       </c>
     </row>
     <row r="25">
@@ -886,7 +988,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>4.682616392771402</v>
+        <v>4.09390926361084</v>
       </c>
     </row>
     <row r="26">
@@ -896,7 +998,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>7.791761557261149</v>
+        <v>4.095109303792318</v>
       </c>
     </row>
     <row r="27">
@@ -906,7 +1008,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>7.858033974965412</v>
+        <v>7.55076805750529</v>
       </c>
     </row>
   </sheetData>
@@ -1530,14 +1632,14 @@
       </c>
       <c r="V4" s="15" t="inlineStr">
         <is>
-          <t>[0, 13, 11, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="W4" s="16" t="n">
         <v>2421</v>
       </c>
       <c r="X4" s="17" t="n">
-        <v>74.29763934338189</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="Y4" s="15" t="b">
         <v>1</v>
@@ -1606,14 +1708,14 @@
       </c>
       <c r="AR4" s="18" t="inlineStr">
         <is>
-          <t>[0, 13, 11, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="AS4" s="19" t="n">
         <v>2421</v>
       </c>
       <c r="AT4" s="20" t="n">
-        <v>74.29763934338189</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="AU4" s="18" t="b">
         <v>1</v>
@@ -1698,14 +1800,14 @@
       </c>
       <c r="N5" s="15" t="inlineStr">
         <is>
-          <t>[0, 16, 1, 15, 0]</t>
+          <t>[0, 11, 13, 15, 0]</t>
         </is>
       </c>
       <c r="O5" s="16" t="n">
-        <v>2968</v>
+        <v>3074</v>
       </c>
       <c r="P5" s="17" t="n">
-        <v>73.83180399377221</v>
+        <v>76.91766635133968</v>
       </c>
       <c r="Q5" s="15" t="b">
         <v>1</v>
@@ -1745,7 +1847,7 @@
         <v>15.97267404033832</v>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>3.448275862068965</v>
+        <v>0</v>
       </c>
       <c r="AC5" s="5" t="n">
         <v>0</v>
@@ -1922,14 +2024,14 @@
       </c>
       <c r="V6" s="15" t="inlineStr">
         <is>
-          <t>[0, 13, 11, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="W6" s="16" t="n">
-        <v>2541</v>
+        <v>2486</v>
       </c>
       <c r="X6" s="17" t="n">
-        <v>74.29763934338189</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="Y6" s="15" t="b">
         <v>1</v>
@@ -1947,7 +2049,7 @@
         <v>0</v>
       </c>
       <c r="AD6" s="5" t="n">
-        <v>36.01108033240997</v>
+        <v>37.39612188365651</v>
       </c>
       <c r="AE6" s="18" t="inlineStr">
         <is>
@@ -1998,14 +2100,14 @@
       </c>
       <c r="AR6" s="18" t="inlineStr">
         <is>
-          <t>[0, 13, 11, 15, 0]</t>
+          <t>[0, 13, 1, 0]</t>
         </is>
       </c>
       <c r="AS6" s="19" t="n">
-        <v>2541</v>
+        <v>2486</v>
       </c>
       <c r="AT6" s="20" t="n">
-        <v>74.29763934338189</v>
+        <v>76.65434719173314</v>
       </c>
       <c r="AU6" s="18" t="b">
         <v>1</v>
@@ -2034,7 +2136,7 @@
         <v>0</v>
       </c>
       <c r="BC6" s="5" t="n">
-        <v>36.01108033240997</v>
+        <v>37.39612188365651</v>
       </c>
       <c r="BD6" s="5" t="n">
         <v>29.28733316544951</v>
@@ -2090,14 +2192,14 @@
       </c>
       <c r="N7" s="15" t="inlineStr">
         <is>
-          <t>[1, 16, 12, 13, 11, 1]</t>
+          <t>[1, 12, 17, 11, 13, 1]</t>
         </is>
       </c>
       <c r="O7" s="16" t="n">
-        <v>3597</v>
+        <v>3949</v>
       </c>
       <c r="P7" s="17" t="n">
-        <v>74.81627471030708</v>
+        <v>70.51893234490386</v>
       </c>
       <c r="Q7" s="15" t="b">
         <v>1</v>
@@ -2137,7 +2239,7 @@
         <v>8.938971891618133</v>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>8.913649025069638</v>
+        <v>0</v>
       </c>
       <c r="AC7" s="5" t="n">
         <v>8.913649025069638</v>
@@ -2314,14 +2416,14 @@
       </c>
       <c r="V8" s="15" t="inlineStr">
         <is>
-          <t>[1, 13, 11, 15, 1]</t>
+          <t>[1, 13, 0, 1]</t>
         </is>
       </c>
       <c r="W8" s="16" t="n">
-        <v>2657</v>
+        <v>2897</v>
       </c>
       <c r="X8" s="17" t="n">
-        <v>68.48294889595655</v>
+        <v>76.65520631352818</v>
       </c>
       <c r="Y8" s="15" t="b">
         <v>1</v>
@@ -2339,7 +2441,7 @@
         <v>23.63420427553444</v>
       </c>
       <c r="AD8" s="5" t="n">
-        <v>47.40696753760887</v>
+        <v>42.65637371338084</v>
       </c>
       <c r="AE8" s="18" t="inlineStr">
         <is>
@@ -2390,14 +2492,14 @@
       </c>
       <c r="AR8" s="18" t="inlineStr">
         <is>
-          <t>[1, 13, 11, 15, 1]</t>
+          <t>[1, 13, 0, 1]</t>
         </is>
       </c>
       <c r="AS8" s="19" t="n">
-        <v>2657</v>
+        <v>2897</v>
       </c>
       <c r="AT8" s="20" t="n">
-        <v>68.48294889595655</v>
+        <v>76.65520631352818</v>
       </c>
       <c r="AU8" s="18" t="b">
         <v>1</v>
@@ -2426,7 +2528,7 @@
         <v>23.63420427553444</v>
       </c>
       <c r="BC8" s="5" t="n">
-        <v>47.40696753760887</v>
+        <v>42.65637371338084</v>
       </c>
       <c r="BD8" s="5" t="n">
         <v>22.0110847189232</v>
@@ -2510,14 +2612,14 @@
       </c>
       <c r="V9" s="15" t="inlineStr">
         <is>
-          <t>[1, 13, 15, 1]</t>
+          <t>[1, 13, 0, 1]</t>
         </is>
       </c>
       <c r="W9" s="16" t="n">
-        <v>2495</v>
+        <v>3038</v>
       </c>
       <c r="X9" s="17" t="n">
-        <v>68.53867309033339</v>
+        <v>76.65520631352818</v>
       </c>
       <c r="Y9" s="15" t="b">
         <v>1</v>
@@ -2535,7 +2637,7 @@
         <v>0</v>
       </c>
       <c r="AD9" s="5" t="n">
-        <v>46.44773556557201</v>
+        <v>34.7928740072977</v>
       </c>
       <c r="AE9" s="18" t="inlineStr">
         <is>
@@ -2586,14 +2688,14 @@
       </c>
       <c r="AR9" s="18" t="inlineStr">
         <is>
-          <t>[1, 13, 15, 1]</t>
+          <t>[1, 13, 0, 1]</t>
         </is>
       </c>
       <c r="AS9" s="19" t="n">
-        <v>2495</v>
+        <v>3038</v>
       </c>
       <c r="AT9" s="20" t="n">
-        <v>68.53867309033339</v>
+        <v>76.65520631352818</v>
       </c>
       <c r="AU9" s="18" t="b">
         <v>1</v>
@@ -2622,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="BC9" s="5" t="n">
-        <v>46.44773556557201</v>
+        <v>34.7928740072977</v>
       </c>
       <c r="BD9" s="5" t="n">
         <v>17.38570508692853</v>
@@ -3070,14 +3172,14 @@
       </c>
       <c r="N12" s="15" t="inlineStr">
         <is>
-          <t>[2, 18, 1, 13, 2]</t>
+          <t>[2, 18, 1, 13, 8, 2]</t>
         </is>
       </c>
       <c r="O12" s="16" t="n">
-        <v>5108</v>
+        <v>5743</v>
       </c>
       <c r="P12" s="17" t="n">
-        <v>71.62834258031488</v>
+        <v>76.231836126931</v>
       </c>
       <c r="Q12" s="15" t="b">
         <v>1</v>
@@ -3098,14 +3200,14 @@
       </c>
       <c r="V12" s="15" t="inlineStr">
         <is>
-          <t>[2, 6, 11, 13, 2]</t>
+          <t>[2, 6, 13, 2]</t>
         </is>
       </c>
       <c r="W12" s="16" t="n">
-        <v>3662</v>
+        <v>2757</v>
       </c>
       <c r="X12" s="17" t="n">
-        <v>72.99489863839968</v>
+        <v>72.73457894316756</v>
       </c>
       <c r="Y12" s="15" t="b">
         <v>1</v>
@@ -3117,13 +3219,13 @@
         <v>0</v>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>11.05693888211736</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AD12" s="5" t="n">
-        <v>36.23541702942713</v>
+        <v>51.99373149921643</v>
       </c>
       <c r="AE12" s="18" t="inlineStr">
         <is>
@@ -3490,14 +3592,14 @@
       </c>
       <c r="V14" s="15" t="inlineStr">
         <is>
-          <t>[3, 4, 10, 3]</t>
+          <t>[3, 4, 14, 3]</t>
         </is>
       </c>
       <c r="W14" s="16" t="n">
-        <v>921</v>
+        <v>3549</v>
       </c>
       <c r="X14" s="17" t="n">
-        <v>69.40688705353338</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="Y14" s="15" t="b">
         <v>1</v>
@@ -3515,7 +3617,7 @@
         <v>0</v>
       </c>
       <c r="AD14" s="5" t="n">
-        <v>74.04902789518174</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="18" t="inlineStr">
         <is>
@@ -3566,14 +3668,14 @@
       </c>
       <c r="AR14" s="18" t="inlineStr">
         <is>
-          <t>[3, 4, 10, 3]</t>
+          <t>[3, 4, 14, 3]</t>
         </is>
       </c>
       <c r="AS14" s="19" t="n">
-        <v>921</v>
+        <v>3549</v>
       </c>
       <c r="AT14" s="20" t="n">
-        <v>69.40688705353338</v>
+        <v>63.4815652406223</v>
       </c>
       <c r="AU14" s="18" t="b">
         <v>1</v>
@@ -3602,7 +3704,7 @@
         <v>0</v>
       </c>
       <c r="BC14" s="5" t="n">
-        <v>74.04902789518174</v>
+        <v>0</v>
       </c>
       <c r="BD14" s="5" t="n">
         <v>0</v>
@@ -4470,14 +4572,14 @@
       </c>
       <c r="V19" s="15" t="inlineStr">
         <is>
-          <t>[5, 14, 4, 5]</t>
+          <t>[5, 14, 3, 5]</t>
         </is>
       </c>
       <c r="W19" s="16" t="n">
-        <v>2796</v>
+        <v>1724</v>
       </c>
       <c r="X19" s="17" t="n">
-        <v>72.12551059405325</v>
+        <v>73.22606566043079</v>
       </c>
       <c r="Y19" s="15" t="b">
         <v>1</v>
@@ -4495,7 +4597,7 @@
         <v>0</v>
       </c>
       <c r="AD19" s="5" t="n">
-        <v>7.417218543046358</v>
+        <v>42.91390728476821</v>
       </c>
       <c r="AE19" s="18" t="inlineStr">
         <is>
@@ -4546,14 +4648,14 @@
       </c>
       <c r="AR19" s="18" t="inlineStr">
         <is>
-          <t>[5, 14, 4, 5]</t>
+          <t>[5, 14, 3, 5]</t>
         </is>
       </c>
       <c r="AS19" s="19" t="n">
-        <v>2796</v>
+        <v>1724</v>
       </c>
       <c r="AT19" s="20" t="n">
-        <v>72.12551059405325</v>
+        <v>73.22606566043079</v>
       </c>
       <c r="AU19" s="18" t="b">
         <v>1</v>
@@ -4582,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="BC19" s="5" t="n">
-        <v>7.417218543046358</v>
+        <v>42.91390728476821</v>
       </c>
       <c r="BD19" s="5" t="n">
         <v>0</v>
@@ -4938,14 +5040,14 @@
       </c>
       <c r="AR21" s="18" t="inlineStr">
         <is>
-          <t>[5, 14, 19, 5]</t>
+          <t>[5, 14, 3, 5]</t>
         </is>
       </c>
       <c r="AS21" s="19" t="n">
-        <v>2164</v>
+        <v>1616</v>
       </c>
       <c r="AT21" s="20" t="n">
-        <v>75.84533600861731</v>
+        <v>73.22606566043079</v>
       </c>
       <c r="AU21" s="18" t="b">
         <v>1</v>
@@ -4974,7 +5076,7 @@
         <v>0</v>
       </c>
       <c r="BC21" s="5" t="n">
-        <v>25.58459422283356</v>
+        <v>44.42916093535076</v>
       </c>
       <c r="BD21" s="5" t="n">
         <v>0</v>
@@ -5058,14 +5160,14 @@
       </c>
       <c r="V22" s="15" t="inlineStr">
         <is>
-          <t>[6, 15, 8, 6]</t>
+          <t>[6, 15, 1, 13, 11, 6]</t>
         </is>
       </c>
       <c r="W22" s="16" t="n">
-        <v>-653</v>
+        <v>3803</v>
       </c>
       <c r="X22" s="17" t="n">
-        <v>75.33210284052421</v>
+        <v>76.04274869886203</v>
       </c>
       <c r="Y22" s="15" t="b">
         <v>1</v>
@@ -5083,7 +5185,7 @@
         <v>0</v>
       </c>
       <c r="AD22" s="5" t="n">
-        <v>116.552598225602</v>
+        <v>3.599493029150823</v>
       </c>
       <c r="AE22" s="18" t="inlineStr">
         <is>
@@ -5134,14 +5236,14 @@
       </c>
       <c r="AR22" s="18" t="inlineStr">
         <is>
-          <t>[6, 15, 0, 11, 6]</t>
+          <t>[6, 15, 1, 13, 11, 6]</t>
         </is>
       </c>
       <c r="AS22" s="19" t="n">
-        <v>2565</v>
+        <v>3803</v>
       </c>
       <c r="AT22" s="20" t="n">
-        <v>63.29161624057945</v>
+        <v>76.04274869886203</v>
       </c>
       <c r="AU22" s="18" t="b">
         <v>1</v>
@@ -5170,7 +5272,7 @@
         <v>0.7625558769392584</v>
       </c>
       <c r="BC22" s="5" t="n">
-        <v>32.55324743623455</v>
+        <v>0</v>
       </c>
       <c r="BD22" s="5" t="n">
         <v>0</v>
@@ -5450,14 +5552,14 @@
       </c>
       <c r="V24" s="15" t="inlineStr">
         <is>
-          <t>[6, 12, 13, 11, 6]</t>
+          <t>[6, 12, 17, 11, 6]</t>
         </is>
       </c>
       <c r="W24" s="16" t="n">
-        <v>2542</v>
+        <v>2035</v>
       </c>
       <c r="X24" s="17" t="n">
-        <v>75.30202355423859</v>
+        <v>76.25021558656204</v>
       </c>
       <c r="Y24" s="15" t="b">
         <v>1</v>
@@ -5475,7 +5577,7 @@
         <v>0</v>
       </c>
       <c r="AD24" s="5" t="n">
-        <v>29.74018794914317</v>
+        <v>43.7534549474848</v>
       </c>
       <c r="AE24" s="18" t="inlineStr">
         <is>
@@ -5526,14 +5628,14 @@
       </c>
       <c r="AR24" s="18" t="inlineStr">
         <is>
-          <t>[6, 12, 13, 11, 6]</t>
+          <t>[6, 12, 17, 11, 6]</t>
         </is>
       </c>
       <c r="AS24" s="19" t="n">
-        <v>2542</v>
+        <v>2035</v>
       </c>
       <c r="AT24" s="20" t="n">
-        <v>75.30202355423859</v>
+        <v>76.25021558656204</v>
       </c>
       <c r="AU24" s="18" t="b">
         <v>1</v>
@@ -5562,7 +5664,7 @@
         <v>0</v>
       </c>
       <c r="BC24" s="5" t="n">
-        <v>29.74018794914317</v>
+        <v>43.7534549474848</v>
       </c>
       <c r="BD24" s="5" t="n">
         <v>0</v>
@@ -5842,14 +5944,14 @@
       </c>
       <c r="V26" s="15" t="inlineStr">
         <is>
-          <t>[7, 13, 11, 6, 7]</t>
+          <t>[7, 13, 6, 7]</t>
         </is>
       </c>
       <c r="W26" s="16" t="n">
-        <v>2741</v>
+        <v>2222</v>
       </c>
       <c r="X26" s="17" t="n">
-        <v>65.84630455243327</v>
+        <v>65.61883663220416</v>
       </c>
       <c r="Y26" s="15" t="b">
         <v>1</v>
@@ -5867,7 +5969,7 @@
         <v>0</v>
       </c>
       <c r="AD26" s="5" t="n">
-        <v>3.007784854918613</v>
+        <v>21.37296532200991</v>
       </c>
       <c r="AE26" s="18" t="inlineStr">
         <is>
@@ -5918,14 +6020,14 @@
       </c>
       <c r="AR26" s="18" t="inlineStr">
         <is>
-          <t>[7, 13, 11, 6, 7]</t>
+          <t>[7, 13, 6, 7]</t>
         </is>
       </c>
       <c r="AS26" s="19" t="n">
-        <v>2741</v>
+        <v>2222</v>
       </c>
       <c r="AT26" s="20" t="n">
-        <v>65.84630455243327</v>
+        <v>65.61883663220416</v>
       </c>
       <c r="AU26" s="18" t="b">
         <v>1</v>
@@ -5954,7 +6056,7 @@
         <v>0</v>
       </c>
       <c r="BC26" s="5" t="n">
-        <v>3.007784854918613</v>
+        <v>21.37296532200991</v>
       </c>
       <c r="BD26" s="5" t="n">
         <v>0</v>
@@ -6038,14 +6140,14 @@
       </c>
       <c r="V27" s="15" t="inlineStr">
         <is>
-          <t>[7, 11, 15, 6, 7]</t>
+          <t>[7, 11, 13, 6, 7]</t>
         </is>
       </c>
       <c r="W27" s="16" t="n">
-        <v>214</v>
+        <v>-4</v>
       </c>
       <c r="X27" s="17" t="n">
-        <v>73.3549742462673</v>
+        <v>68.23810542118596</v>
       </c>
       <c r="Y27" s="15" t="b">
         <v>1</v>
@@ -6063,7 +6165,7 @@
         <v>0</v>
       </c>
       <c r="AD27" s="5" t="n">
-        <v>90.80756013745705</v>
+        <v>100.1718213058419</v>
       </c>
       <c r="AE27" s="18" t="inlineStr">
         <is>
@@ -6114,14 +6216,14 @@
       </c>
       <c r="AR27" s="18" t="inlineStr">
         <is>
-          <t>[7, 11, 15, 7]</t>
+          <t>[7, 11, 13, 6, 7]</t>
         </is>
       </c>
       <c r="AS27" s="19" t="n">
-        <v>1225</v>
+        <v>-4</v>
       </c>
       <c r="AT27" s="20" t="n">
-        <v>71.35147682744685</v>
+        <v>68.23810542118596</v>
       </c>
       <c r="AU27" s="18" t="b">
         <v>1</v>
@@ -6150,7 +6252,7 @@
         <v>0</v>
       </c>
       <c r="BC27" s="5" t="n">
-        <v>47.37972508591065</v>
+        <v>100.1718213058419</v>
       </c>
       <c r="BD27" s="5" t="n">
         <v>0</v>
@@ -6206,14 +6308,14 @@
       </c>
       <c r="N28" s="15" t="inlineStr">
         <is>
-          <t>[8, 18, 17, 1, 13, 8]</t>
+          <t>[8, 18, 2, 11, 13, 8]</t>
         </is>
       </c>
       <c r="O28" s="16" t="n">
-        <v>4097</v>
+        <v>4067</v>
       </c>
       <c r="P28" s="17" t="n">
-        <v>76.36987251988171</v>
+        <v>71.86492405207225</v>
       </c>
       <c r="Q28" s="15" t="b">
         <v>1</v>
@@ -6253,7 +6355,7 @@
         <v>0</v>
       </c>
       <c r="AB28" s="5" t="n">
-        <v>0</v>
+        <v>0.7322431047107639</v>
       </c>
       <c r="AC28" s="5" t="n">
         <v>0</v>
@@ -6430,14 +6532,14 @@
       </c>
       <c r="V29" s="15" t="inlineStr">
         <is>
-          <t>[8, 18, 2, 11, 13, 8]</t>
+          <t>[8, 18, 11, 13, 8]</t>
         </is>
       </c>
       <c r="W29" s="16" t="n">
-        <v>2518</v>
+        <v>2564</v>
       </c>
       <c r="X29" s="17" t="n">
-        <v>71.86492405207225</v>
+        <v>68.17985665164061</v>
       </c>
       <c r="Y29" s="15" t="b">
         <v>1</v>
@@ -6455,7 +6557,7 @@
         <v>2.922990444069702</v>
       </c>
       <c r="AD29" s="5" t="n">
-        <v>29.22990444069702</v>
+        <v>27.93704328274311</v>
       </c>
       <c r="AE29" s="18" t="inlineStr">
         <is>
@@ -6506,14 +6608,14 @@
       </c>
       <c r="AR29" s="18" t="inlineStr">
         <is>
-          <t>[8, 18, 2, 11, 13, 8]</t>
+          <t>[8, 18, 11, 13, 8]</t>
         </is>
       </c>
       <c r="AS29" s="19" t="n">
-        <v>2518</v>
+        <v>2564</v>
       </c>
       <c r="AT29" s="20" t="n">
-        <v>71.86492405207225</v>
+        <v>68.17985665164061</v>
       </c>
       <c r="AU29" s="18" t="b">
         <v>1</v>
@@ -6542,7 +6644,7 @@
         <v>2.922990444069702</v>
       </c>
       <c r="BC29" s="5" t="n">
-        <v>29.22990444069702</v>
+        <v>27.93704328274311</v>
       </c>
       <c r="BD29" s="5" t="n">
         <v>27.93704328274311</v>
@@ -6626,14 +6728,14 @@
       </c>
       <c r="V30" s="15" t="inlineStr">
         <is>
-          <t>[8, 11, 18, 2, 8]</t>
+          <t>[8, 11, 13, 17, 2, 8]</t>
         </is>
       </c>
       <c r="W30" s="16" t="n">
-        <v>1585</v>
+        <v>3312</v>
       </c>
       <c r="X30" s="17" t="n">
-        <v>65.41050549960794</v>
+        <v>75.03404125883236</v>
       </c>
       <c r="Y30" s="15" t="b">
         <v>1</v>
@@ -6651,7 +6753,7 @@
         <v>4.404622341316363</v>
       </c>
       <c r="AD30" s="5" t="n">
-        <v>73.45503265784626</v>
+        <v>44.53190420365098</v>
       </c>
       <c r="AE30" s="18" t="inlineStr">
         <is>
@@ -6702,14 +6804,14 @@
       </c>
       <c r="AR30" s="18" t="inlineStr">
         <is>
-          <t>[8, 11, 18, 2, 8]</t>
+          <t>[8, 11, 13, 17, 2, 8]</t>
         </is>
       </c>
       <c r="AS30" s="19" t="n">
-        <v>1585</v>
+        <v>3312</v>
       </c>
       <c r="AT30" s="20" t="n">
-        <v>65.41050549960794</v>
+        <v>75.03404125883236</v>
       </c>
       <c r="AU30" s="18" t="b">
         <v>1</v>
@@ -6738,7 +6840,7 @@
         <v>4.404622341316363</v>
       </c>
       <c r="BC30" s="5" t="n">
-        <v>73.45503265784626</v>
+        <v>44.53190420365098</v>
       </c>
       <c r="BD30" s="5" t="n">
         <v>4.404622341316363</v>
@@ -7802,14 +7904,14 @@
       </c>
       <c r="V36" s="15" t="inlineStr">
         <is>
-          <t>[10, 4, 14, 10]</t>
+          <t>[10, 4, 3, 10]</t>
         </is>
       </c>
       <c r="W36" s="16" t="n">
-        <v>-182</v>
+        <v>-600</v>
       </c>
       <c r="X36" s="17" t="n">
-        <v>64.55122978877812</v>
+        <v>69.66899203815812</v>
       </c>
       <c r="Y36" s="15" t="b">
         <v>1</v>
@@ -7827,7 +7929,7 @@
         <v>25.80645161290322</v>
       </c>
       <c r="AD36" s="5" t="n">
-        <v>117.7908113391984</v>
+        <v>158.6510263929619</v>
       </c>
       <c r="AE36" s="18" t="inlineStr">
         <is>
@@ -7878,14 +7980,14 @@
       </c>
       <c r="AR36" s="18" t="inlineStr">
         <is>
-          <t>[10, 4, 14, 10]</t>
+          <t>[10, 4, 3, 10]</t>
         </is>
       </c>
       <c r="AS36" s="19" t="n">
-        <v>-182</v>
+        <v>-600</v>
       </c>
       <c r="AT36" s="20" t="n">
-        <v>64.55122978877812</v>
+        <v>69.66899203815812</v>
       </c>
       <c r="AU36" s="18" t="b">
         <v>1</v>
@@ -7914,7 +8016,7 @@
         <v>25.80645161290322</v>
       </c>
       <c r="BC36" s="5" t="n">
-        <v>117.7908113391984</v>
+        <v>158.6510263929619</v>
       </c>
       <c r="BD36" s="5" t="n">
         <v>25.80645161290322</v>
@@ -8194,14 +8296,14 @@
       </c>
       <c r="V38" s="15" t="inlineStr">
         <is>
-          <t>[11, 13, 12, 16, 1, 11]</t>
+          <t>[11, 13, 7, 6, 11]</t>
         </is>
       </c>
       <c r="W38" s="16" t="n">
-        <v>3252</v>
+        <v>3452</v>
       </c>
       <c r="X38" s="17" t="n">
-        <v>74.80342441332024</v>
+        <v>65.89413159769893</v>
       </c>
       <c r="Y38" s="15" t="b">
         <v>1</v>
@@ -8219,7 +8321,7 @@
         <v>0</v>
       </c>
       <c r="AD38" s="5" t="n">
-        <v>26.75675675675675</v>
+        <v>22.25225225225225</v>
       </c>
       <c r="AE38" s="18" t="inlineStr">
         <is>
@@ -8270,14 +8372,14 @@
       </c>
       <c r="AR38" s="18" t="inlineStr">
         <is>
-          <t>[11, 13, 12, 16, 1, 11]</t>
+          <t>[11, 13, 7, 6, 11]</t>
         </is>
       </c>
       <c r="AS38" s="19" t="n">
-        <v>3252</v>
+        <v>3452</v>
       </c>
       <c r="AT38" s="20" t="n">
-        <v>74.80342441332024</v>
+        <v>65.89413159769893</v>
       </c>
       <c r="AU38" s="18" t="b">
         <v>1</v>
@@ -8306,7 +8408,7 @@
         <v>0</v>
       </c>
       <c r="BC38" s="5" t="n">
-        <v>26.75675675675675</v>
+        <v>22.25225225225225</v>
       </c>
       <c r="BD38" s="5" t="n">
         <v>18.33333333333333</v>
@@ -8390,14 +8492,14 @@
       </c>
       <c r="V39" s="15" t="inlineStr">
         <is>
-          <t>[11, 16, 17, 11]</t>
+          <t>[11, 16, 12, 17, 11]</t>
         </is>
       </c>
       <c r="W39" s="16" t="n">
-        <v>1754</v>
+        <v>2491</v>
       </c>
       <c r="X39" s="17" t="n">
-        <v>73.8088571780594</v>
+        <v>75.58359765984289</v>
       </c>
       <c r="Y39" s="15" t="b">
         <v>1</v>
@@ -8415,7 +8517,7 @@
         <v>0</v>
       </c>
       <c r="AD39" s="5" t="n">
-        <v>57.7145612343298</v>
+        <v>39.94696239151398</v>
       </c>
       <c r="AE39" s="18" t="inlineStr">
         <is>
@@ -8466,14 +8568,14 @@
       </c>
       <c r="AR39" s="18" t="inlineStr">
         <is>
-          <t>[11, 16, 17, 11]</t>
+          <t>[11, 16, 12, 17, 11]</t>
         </is>
       </c>
       <c r="AS39" s="19" t="n">
-        <v>1754</v>
+        <v>2491</v>
       </c>
       <c r="AT39" s="20" t="n">
-        <v>73.8088571780594</v>
+        <v>75.58359765984289</v>
       </c>
       <c r="AU39" s="18" t="b">
         <v>1</v>
@@ -8502,7 +8604,7 @@
         <v>0</v>
       </c>
       <c r="BC39" s="5" t="n">
-        <v>57.7145612343298</v>
+        <v>39.94696239151398</v>
       </c>
       <c r="BD39" s="5" t="n">
         <v>23.33654773384764</v>
@@ -8586,14 +8688,14 @@
       </c>
       <c r="V40" s="15" t="inlineStr">
         <is>
-          <t>[12, 16, 17, 13, 1, 12]</t>
+          <t>[12, 16, 11, 13, 12]</t>
         </is>
       </c>
       <c r="W40" s="16" t="n">
-        <v>3773</v>
+        <v>3796</v>
       </c>
       <c r="X40" s="17" t="n">
-        <v>71.05017633208588</v>
+        <v>74.66154658545187</v>
       </c>
       <c r="Y40" s="15" t="b">
         <v>1</v>
@@ -8611,7 +8713,7 @@
         <v>6.360642239604776</v>
       </c>
       <c r="AD40" s="5" t="n">
-        <v>22.3342939481268</v>
+        <v>21.86084808563195</v>
       </c>
       <c r="AE40" s="18" t="inlineStr">
         <is>
@@ -8662,14 +8764,14 @@
       </c>
       <c r="AR40" s="18" t="inlineStr">
         <is>
-          <t>[12, 16, 17, 13, 1, 12]</t>
+          <t>[12, 16, 11, 13, 12]</t>
         </is>
       </c>
       <c r="AS40" s="19" t="n">
-        <v>3773</v>
+        <v>3796</v>
       </c>
       <c r="AT40" s="20" t="n">
-        <v>71.05017633208588</v>
+        <v>74.66154658545187</v>
       </c>
       <c r="AU40" s="18" t="b">
         <v>1</v>
@@ -8698,7 +8800,7 @@
         <v>6.360642239604776</v>
       </c>
       <c r="BC40" s="5" t="n">
-        <v>22.3342939481268</v>
+        <v>21.86084808563195</v>
       </c>
       <c r="BD40" s="5" t="n">
         <v>6.360642239604776</v>
@@ -8782,14 +8884,14 @@
       </c>
       <c r="V41" s="15" t="inlineStr">
         <is>
-          <t>[12, 13, 11, 16, 12]</t>
+          <t>[12, 13, 16, 1, 12]</t>
         </is>
       </c>
       <c r="W41" s="16" t="n">
-        <v>3064</v>
+        <v>3043</v>
       </c>
       <c r="X41" s="17" t="n">
-        <v>74.63540562751945</v>
+        <v>72.03869630325187</v>
       </c>
       <c r="Y41" s="15" t="b">
         <v>1</v>
@@ -8807,7 +8909,7 @@
         <v>7.766749379652606</v>
       </c>
       <c r="AD41" s="5" t="n">
-        <v>23.97022332506203</v>
+        <v>24.49131513647643</v>
       </c>
       <c r="AE41" s="18" t="inlineStr">
         <is>
@@ -8858,14 +8960,14 @@
       </c>
       <c r="AR41" s="18" t="inlineStr">
         <is>
-          <t>[12, 13, 11, 16, 12]</t>
+          <t>[12, 13, 16, 1, 12]</t>
         </is>
       </c>
       <c r="AS41" s="19" t="n">
-        <v>3064</v>
+        <v>3043</v>
       </c>
       <c r="AT41" s="20" t="n">
-        <v>74.63540562751945</v>
+        <v>72.03869630325187</v>
       </c>
       <c r="AU41" s="18" t="b">
         <v>1</v>
@@ -8894,7 +8996,7 @@
         <v>0</v>
       </c>
       <c r="BC41" s="5" t="n">
-        <v>17.56793112725316</v>
+        <v>18.13290287866559</v>
       </c>
       <c r="BD41" s="5" t="n">
         <v>4.250739843960183</v>
@@ -8978,14 +9080,14 @@
       </c>
       <c r="V42" s="15" t="inlineStr">
         <is>
-          <t>[12, 15, 17, 12]</t>
+          <t>[12, 15, 16, 12]</t>
         </is>
       </c>
       <c r="W42" s="16" t="n">
-        <v>2081</v>
+        <v>2479</v>
       </c>
       <c r="X42" s="17" t="n">
-        <v>73.50842360051703</v>
+        <v>71.33989906424667</v>
       </c>
       <c r="Y42" s="15" t="b">
         <v>1</v>
@@ -9003,7 +9105,7 @@
         <v>2.618933205189813</v>
       </c>
       <c r="AD42" s="5" t="n">
-        <v>50</v>
+        <v>40.43728976453628</v>
       </c>
       <c r="AE42" s="18" t="inlineStr">
         <is>
@@ -9054,14 +9156,14 @@
       </c>
       <c r="AR42" s="18" t="inlineStr">
         <is>
-          <t>[12, 15, 17, 12]</t>
+          <t>[12, 15, 16, 12]</t>
         </is>
       </c>
       <c r="AS42" s="19" t="n">
-        <v>2081</v>
+        <v>2479</v>
       </c>
       <c r="AT42" s="20" t="n">
-        <v>73.50842360051703</v>
+        <v>71.33989906424667</v>
       </c>
       <c r="AU42" s="18" t="b">
         <v>1</v>
@@ -9090,7 +9192,7 @@
         <v>2.618933205189813</v>
       </c>
       <c r="BC42" s="5" t="n">
-        <v>50</v>
+        <v>40.43728976453628</v>
       </c>
       <c r="BD42" s="5" t="n">
         <v>8.721768380586257</v>
@@ -9370,14 +9472,14 @@
       </c>
       <c r="V44" s="15" t="inlineStr">
         <is>
-          <t>[13, 7, 6, 11, 13]</t>
+          <t>[13, 7, 11, 13]</t>
         </is>
       </c>
       <c r="W44" s="16" t="n">
-        <v>3585</v>
+        <v>3075</v>
       </c>
       <c r="X44" s="17" t="n">
-        <v>65.89413159769894</v>
+        <v>64.95063789465291</v>
       </c>
       <c r="Y44" s="15" t="b">
         <v>1</v>
@@ -9395,7 +9497,7 @@
         <v>2.630297126156843</v>
       </c>
       <c r="AD44" s="5" t="n">
-        <v>12.68874817340477</v>
+        <v>25.10959571358987</v>
       </c>
       <c r="AE44" s="18" t="inlineStr">
         <is>
@@ -9446,14 +9548,14 @@
       </c>
       <c r="AR44" s="18" t="inlineStr">
         <is>
-          <t>[13, 7, 6, 11, 13]</t>
+          <t>[13, 7, 11, 13]</t>
         </is>
       </c>
       <c r="AS44" s="19" t="n">
-        <v>3585</v>
+        <v>3075</v>
       </c>
       <c r="AT44" s="20" t="n">
-        <v>65.89413159769894</v>
+        <v>64.95063789465291</v>
       </c>
       <c r="AU44" s="18" t="b">
         <v>1</v>
@@ -9482,7 +9584,7 @@
         <v>2.630297126156843</v>
       </c>
       <c r="BC44" s="5" t="n">
-        <v>12.68874817340477</v>
+        <v>25.10959571358987</v>
       </c>
       <c r="BD44" s="5" t="n">
         <v>0</v>
@@ -9538,14 +9640,14 @@
       </c>
       <c r="N45" s="15" t="inlineStr">
         <is>
-          <t>[13, 2, 11, 8, 13]</t>
+          <t>[13, 1, 17, 18, 2, 8, 13]</t>
         </is>
       </c>
       <c r="O45" s="16" t="n">
-        <v>4117</v>
+        <v>4676</v>
       </c>
       <c r="P45" s="17" t="n">
-        <v>74.33466845054575</v>
+        <v>76.92379758974532</v>
       </c>
       <c r="Q45" s="15" t="b">
         <v>1</v>
@@ -9566,14 +9668,14 @@
       </c>
       <c r="V45" s="15" t="inlineStr">
         <is>
-          <t>[13, 6, 2, 13]</t>
+          <t>[13, 6, 12, 13]</t>
         </is>
       </c>
       <c r="W45" s="16" t="n">
-        <v>2336</v>
+        <v>2943</v>
       </c>
       <c r="X45" s="17" t="n">
-        <v>72.7077091684051</v>
+        <v>75.07455563400949</v>
       </c>
       <c r="Y45" s="15" t="b">
         <v>1</v>
@@ -9585,13 +9687,13 @@
         <v>12.55346449957228</v>
       </c>
       <c r="AB45" s="5" t="n">
-        <v>11.9546621043627</v>
+        <v>0</v>
       </c>
       <c r="AC45" s="5" t="n">
         <v>11.9546621043627</v>
       </c>
       <c r="AD45" s="5" t="n">
-        <v>50.04277159965783</v>
+        <v>37.06159110350727</v>
       </c>
       <c r="AE45" s="18" t="inlineStr">
         <is>
@@ -9642,14 +9744,14 @@
       </c>
       <c r="AR45" s="18" t="inlineStr">
         <is>
-          <t>[13, 6, 2, 13]</t>
+          <t>[13, 6, 12, 13]</t>
         </is>
       </c>
       <c r="AS45" s="19" t="n">
-        <v>2336</v>
+        <v>2943</v>
       </c>
       <c r="AT45" s="20" t="n">
-        <v>72.7077091684051</v>
+        <v>75.07455563400949</v>
       </c>
       <c r="AU45" s="18" t="b">
         <v>1</v>
@@ -9678,7 +9780,7 @@
         <v>11.9546621043627</v>
       </c>
       <c r="BC45" s="5" t="n">
-        <v>50.04277159965783</v>
+        <v>37.06159110350727</v>
       </c>
       <c r="BD45" s="5" t="n">
         <v>14.64927288280582</v>
@@ -9958,14 +10060,14 @@
       </c>
       <c r="V47" s="15" t="inlineStr">
         <is>
-          <t>[14, 5, 19, 14]</t>
+          <t>[14, 5, 4, 14]</t>
         </is>
       </c>
       <c r="W47" s="16" t="n">
-        <v>1740</v>
+        <v>1788</v>
       </c>
       <c r="X47" s="17" t="n">
-        <v>75.83863254208322</v>
+        <v>72.10731512057799</v>
       </c>
       <c r="Y47" s="15" t="b">
         <v>1</v>
@@ -9983,7 +10085,7 @@
         <v>0</v>
       </c>
       <c r="AD47" s="5" t="n">
-        <v>44.5859872611465</v>
+        <v>43.05732484076433</v>
       </c>
       <c r="AE47" s="18" t="inlineStr">
         <is>
@@ -10034,14 +10136,14 @@
       </c>
       <c r="AR47" s="18" t="inlineStr">
         <is>
-          <t>[14, 5, 19, 14]</t>
+          <t>[14, 5, 4, 14]</t>
         </is>
       </c>
       <c r="AS47" s="19" t="n">
-        <v>1740</v>
+        <v>1788</v>
       </c>
       <c r="AT47" s="20" t="n">
-        <v>75.83863254208322</v>
+        <v>72.10731512057799</v>
       </c>
       <c r="AU47" s="18" t="b">
         <v>1</v>
@@ -10070,7 +10172,7 @@
         <v>0</v>
       </c>
       <c r="BC47" s="5" t="n">
-        <v>44.5859872611465</v>
+        <v>43.05732484076433</v>
       </c>
       <c r="BD47" s="5" t="n">
         <v>0</v>
@@ -10350,14 +10452,14 @@
       </c>
       <c r="V49" s="15" t="inlineStr">
         <is>
-          <t>[15, 12, 16, 1, 15]</t>
+          <t>[15, 12, 17, 1, 15]</t>
         </is>
       </c>
       <c r="W49" s="16" t="n">
-        <v>3286</v>
+        <v>3290</v>
       </c>
       <c r="X49" s="17" t="n">
-        <v>74.88985714445482</v>
+        <v>74.91763749476773</v>
       </c>
       <c r="Y49" s="15" t="b">
         <v>1</v>
@@ -10375,7 +10477,7 @@
         <v>0</v>
       </c>
       <c r="AD49" s="5" t="n">
-        <v>21.66865315852205</v>
+        <v>21.57330154946365</v>
       </c>
       <c r="AE49" s="18" t="inlineStr">
         <is>
@@ -10426,14 +10528,14 @@
       </c>
       <c r="AR49" s="18" t="inlineStr">
         <is>
-          <t>[15, 12, 16, 1, 15]</t>
+          <t>[15, 12, 17, 1, 15]</t>
         </is>
       </c>
       <c r="AS49" s="19" t="n">
-        <v>3286</v>
+        <v>3290</v>
       </c>
       <c r="AT49" s="20" t="n">
-        <v>74.88985714445482</v>
+        <v>74.91763749476773</v>
       </c>
       <c r="AU49" s="18" t="b">
         <v>1</v>
@@ -10462,7 +10564,7 @@
         <v>0</v>
       </c>
       <c r="BC49" s="5" t="n">
-        <v>21.66865315852205</v>
+        <v>21.57330154946365</v>
       </c>
       <c r="BD49" s="5" t="n">
         <v>20.66746126340882</v>
@@ -10546,14 +10648,14 @@
       </c>
       <c r="V50" s="15" t="inlineStr">
         <is>
-          <t>[15, 1, 13, 11, 6, 15]</t>
+          <t>[15, 1, 17, 12, 15]</t>
         </is>
       </c>
       <c r="W50" s="16" t="n">
-        <v>3802</v>
+        <v>3239</v>
       </c>
       <c r="X50" s="17" t="n">
-        <v>76.04274869886204</v>
+        <v>74.2320275637102</v>
       </c>
       <c r="Y50" s="15" t="b">
         <v>1</v>
@@ -10571,7 +10673,7 @@
         <v>7.022619673855865</v>
       </c>
       <c r="AD50" s="5" t="n">
-        <v>0</v>
+        <v>14.80799579168858</v>
       </c>
       <c r="AE50" s="18" t="inlineStr">
         <is>
@@ -10622,14 +10724,14 @@
       </c>
       <c r="AR50" s="18" t="inlineStr">
         <is>
-          <t>[15, 1, 13, 11, 6, 15]</t>
+          <t>[15, 1, 17, 12, 15]</t>
         </is>
       </c>
       <c r="AS50" s="19" t="n">
-        <v>3802</v>
+        <v>3239</v>
       </c>
       <c r="AT50" s="20" t="n">
-        <v>76.04274869886204</v>
+        <v>74.2320275637102</v>
       </c>
       <c r="AU50" s="18" t="b">
         <v>1</v>
@@ -10658,7 +10760,7 @@
         <v>7.022619673855865</v>
       </c>
       <c r="BC50" s="5" t="n">
-        <v>0</v>
+        <v>14.80799579168858</v>
       </c>
       <c r="BD50" s="5" t="n">
         <v>7.022619673855865</v>
@@ -10742,14 +10844,14 @@
       </c>
       <c r="V51" s="15" t="inlineStr">
         <is>
-          <t>[15, 12, 16, 1, 15]</t>
+          <t>[15, 12, 17, 1, 15]</t>
         </is>
       </c>
       <c r="W51" s="16" t="n">
-        <v>3035</v>
+        <v>3050</v>
       </c>
       <c r="X51" s="17" t="n">
-        <v>74.88985714445482</v>
+        <v>74.91763749476773</v>
       </c>
       <c r="Y51" s="15" t="b">
         <v>1</v>
@@ -10767,7 +10869,7 @@
         <v>0.7117437722419928</v>
       </c>
       <c r="AD51" s="5" t="n">
-        <v>22.85205897305541</v>
+        <v>22.4707676664972</v>
       </c>
       <c r="AE51" s="18" t="inlineStr">
         <is>
@@ -10818,14 +10920,14 @@
       </c>
       <c r="AR51" s="18" t="inlineStr">
         <is>
-          <t>[15, 12, 16, 1, 15]</t>
+          <t>[15, 12, 17, 1, 15]</t>
         </is>
       </c>
       <c r="AS51" s="19" t="n">
-        <v>3035</v>
+        <v>3050</v>
       </c>
       <c r="AT51" s="20" t="n">
-        <v>74.88985714445482</v>
+        <v>74.91763749476773</v>
       </c>
       <c r="AU51" s="18" t="b">
         <v>1</v>
@@ -10854,7 +10956,7 @@
         <v>0.7117437722419928</v>
       </c>
       <c r="BC51" s="5" t="n">
-        <v>22.85205897305541</v>
+        <v>22.4707676664972</v>
       </c>
       <c r="BD51" s="5" t="n">
         <v>4.47381799694967</v>
@@ -10938,14 +11040,14 @@
       </c>
       <c r="V52" s="15" t="inlineStr">
         <is>
-          <t>[16, 11, 13, 12, 16]</t>
+          <t>[16, 11, 1, 12, 16]</t>
         </is>
       </c>
       <c r="W52" s="16" t="n">
-        <v>3666</v>
+        <v>3145</v>
       </c>
       <c r="X52" s="17" t="n">
-        <v>74.66154658545189</v>
+        <v>68.36687835621275</v>
       </c>
       <c r="Y52" s="15" t="b">
         <v>1</v>
@@ -10963,7 +11065,7 @@
         <v>0</v>
       </c>
       <c r="AD52" s="5" t="n">
-        <v>8.143322475570033</v>
+        <v>21.19769481332999</v>
       </c>
       <c r="AE52" s="18" t="inlineStr">
         <is>
@@ -11014,14 +11116,14 @@
       </c>
       <c r="AR52" s="18" t="inlineStr">
         <is>
-          <t>[16, 11, 13, 12, 16]</t>
+          <t>[16, 11, 1, 12, 16]</t>
         </is>
       </c>
       <c r="AS52" s="19" t="n">
-        <v>3666</v>
+        <v>3145</v>
       </c>
       <c r="AT52" s="20" t="n">
-        <v>74.66154658545189</v>
+        <v>68.36687835621275</v>
       </c>
       <c r="AU52" s="18" t="b">
         <v>1</v>
@@ -11050,7 +11152,7 @@
         <v>0</v>
       </c>
       <c r="BC52" s="5" t="n">
-        <v>8.143322475570033</v>
+        <v>21.19769481332999</v>
       </c>
       <c r="BD52" s="5" t="n">
         <v>0.2004510147832624</v>
@@ -11106,14 +11208,14 @@
       </c>
       <c r="N53" s="15" t="inlineStr">
         <is>
-          <t>[16, 12, 13, 17, 1, 16]</t>
+          <t>[16, 12, 1, 13, 17, 16]</t>
         </is>
       </c>
       <c r="O53" s="16" t="n">
-        <v>4270</v>
+        <v>4463</v>
       </c>
       <c r="P53" s="17" t="n">
-        <v>70.12394837102107</v>
+        <v>71.12444971666353</v>
       </c>
       <c r="Q53" s="15" t="b">
         <v>1</v>
@@ -11134,14 +11236,14 @@
       </c>
       <c r="V53" s="15" t="inlineStr">
         <is>
-          <t>[16, 17, 13, 1, 12, 16]</t>
+          <t>[16, 17, 1, 12, 16]</t>
         </is>
       </c>
       <c r="W53" s="16" t="n">
-        <v>3113</v>
+        <v>2605</v>
       </c>
       <c r="X53" s="17" t="n">
-        <v>71.05017633208588</v>
+        <v>48.92562036480709</v>
       </c>
       <c r="Y53" s="15" t="b">
         <v>1</v>
@@ -11153,13 +11255,13 @@
         <v>17.9027559937262</v>
       </c>
       <c r="AB53" s="5" t="n">
-        <v>4.324445440286802</v>
+        <v>0</v>
       </c>
       <c r="AC53" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AD53" s="5" t="n">
-        <v>30.24871162894914</v>
+        <v>41.63118978265741</v>
       </c>
       <c r="AE53" s="18" t="inlineStr">
         <is>
@@ -11210,14 +11312,14 @@
       </c>
       <c r="AR53" s="18" t="inlineStr">
         <is>
-          <t>[16, 17, 13, 1, 12, 16]</t>
+          <t>[16, 17, 1, 12, 16]</t>
         </is>
       </c>
       <c r="AS53" s="19" t="n">
-        <v>3113</v>
+        <v>2605</v>
       </c>
       <c r="AT53" s="20" t="n">
-        <v>71.05017633208588</v>
+        <v>48.92562036480709</v>
       </c>
       <c r="AU53" s="18" t="b">
         <v>1</v>
@@ -11246,7 +11348,7 @@
         <v>0</v>
       </c>
       <c r="BC53" s="5" t="n">
-        <v>15.0382096069869</v>
+        <v>28.9028384279476</v>
       </c>
       <c r="BD53" s="5" t="n">
         <v>0</v>
@@ -11526,14 +11628,14 @@
       </c>
       <c r="V55" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 1, 13, 17]</t>
+          <t>[17, 16, 11, 17]</t>
         </is>
       </c>
       <c r="W55" s="16" t="n">
-        <v>4081</v>
+        <v>2998</v>
       </c>
       <c r="X55" s="17" t="n">
-        <v>66.0913104072372</v>
+        <v>74.08499656427625</v>
       </c>
       <c r="Y55" s="15" t="b">
         <v>1</v>
@@ -11551,7 +11653,7 @@
         <v>0.8512544802867384</v>
       </c>
       <c r="AD55" s="5" t="n">
-        <v>8.579749103942651</v>
+        <v>32.84050179211469</v>
       </c>
       <c r="AE55" s="18" t="inlineStr">
         <is>
@@ -11602,14 +11704,14 @@
       </c>
       <c r="AR55" s="18" t="inlineStr">
         <is>
-          <t>[17, 16, 1, 13, 17]</t>
+          <t>[17, 16, 11, 17]</t>
         </is>
       </c>
       <c r="AS55" s="19" t="n">
-        <v>4081</v>
+        <v>2998</v>
       </c>
       <c r="AT55" s="20" t="n">
-        <v>66.0913104072372</v>
+        <v>74.08499656427625</v>
       </c>
       <c r="AU55" s="18" t="b">
         <v>1</v>
@@ -11638,7 +11740,7 @@
         <v>0.8512544802867384</v>
       </c>
       <c r="BC55" s="5" t="n">
-        <v>8.579749103942651</v>
+        <v>32.84050179211469</v>
       </c>
       <c r="BD55" s="5" t="n">
         <v>16.71146953405018</v>
@@ -11871,14 +11973,14 @@
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 12, 1, 13, 17]</t>
+          <t>[17, 16, 12, 13, 17]</t>
         </is>
       </c>
       <c r="J57" s="16" t="n">
-        <v>3916</v>
+        <v>3528</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>71.12444971666355</v>
+        <v>67.42434623698556</v>
       </c>
       <c r="L57" s="15" t="b">
         <v>1</v>
@@ -11918,14 +12020,14 @@
       </c>
       <c r="V57" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 1, 12, 17]</t>
+          <t>[17, 16, 13, 17]</t>
         </is>
       </c>
       <c r="W57" s="16" t="n">
-        <v>3078</v>
+        <v>2773</v>
       </c>
       <c r="X57" s="17" t="n">
-        <v>53.32093090327441</v>
+        <v>64.18249569441392</v>
       </c>
       <c r="Y57" s="15" t="b">
         <v>1</v>
@@ -11934,7 +12036,7 @@
         <v>0</v>
       </c>
       <c r="AA57" s="5" t="n">
-        <v>0</v>
+        <v>9.908069458631257</v>
       </c>
       <c r="AB57" s="5" t="n">
         <v>0</v>
@@ -11943,7 +12045,7 @@
         <v>0</v>
       </c>
       <c r="AD57" s="5" t="n">
-        <v>21.39938712972421</v>
+        <v>29.1879468845761</v>
       </c>
       <c r="AE57" s="18" t="inlineStr">
         <is>
@@ -11994,14 +12096,14 @@
       </c>
       <c r="AR57" s="18" t="inlineStr">
         <is>
-          <t>[17, 16, 1, 12, 17]</t>
+          <t>[17, 16, 11, 17]</t>
         </is>
       </c>
       <c r="AS57" s="19" t="n">
-        <v>3078</v>
+        <v>2803</v>
       </c>
       <c r="AT57" s="20" t="n">
-        <v>53.32093090327441</v>
+        <v>74.08499656427625</v>
       </c>
       <c r="AU57" s="18" t="b">
         <v>1</v>
@@ -12030,7 +12132,7 @@
         <v>0</v>
       </c>
       <c r="BC57" s="5" t="n">
-        <v>21.39938712972421</v>
+        <v>28.42185903983657</v>
       </c>
       <c r="BD57" s="5" t="n">
         <v>1.072522982635342</v>
@@ -12310,14 +12412,14 @@
       </c>
       <c r="V59" s="15" t="inlineStr">
         <is>
-          <t>[18, 12, 1, 13, 18]</t>
+          <t>[18, 12, 13, 2, 18]</t>
         </is>
       </c>
       <c r="W59" s="16" t="n">
-        <v>2920</v>
+        <v>3185</v>
       </c>
       <c r="X59" s="17" t="n">
-        <v>76.24604939157767</v>
+        <v>76.02610864345647</v>
       </c>
       <c r="Y59" s="15" t="b">
         <v>1</v>
@@ -12335,7 +12437,7 @@
         <v>14.8460661345496</v>
       </c>
       <c r="AD59" s="5" t="n">
-        <v>33.40935005701255</v>
+        <v>27.3660205245154</v>
       </c>
       <c r="AE59" s="18" t="inlineStr">
         <is>
@@ -12386,14 +12488,14 @@
       </c>
       <c r="AR59" s="18" t="inlineStr">
         <is>
-          <t>[18, 12, 1, 13, 18]</t>
+          <t>[18, 12, 13, 2, 18]</t>
         </is>
       </c>
       <c r="AS59" s="19" t="n">
-        <v>2920</v>
+        <v>3185</v>
       </c>
       <c r="AT59" s="20" t="n">
-        <v>76.24604939157767</v>
+        <v>76.02610864345647</v>
       </c>
       <c r="AU59" s="18" t="b">
         <v>1</v>
@@ -12422,7 +12524,7 @@
         <v>14.8460661345496</v>
       </c>
       <c r="BC59" s="5" t="n">
-        <v>33.40935005701255</v>
+        <v>27.3660205245154</v>
       </c>
       <c r="BD59" s="5" t="n">
         <v>0</v>
@@ -12478,14 +12580,14 @@
       </c>
       <c r="N60" s="15" t="inlineStr">
         <is>
-          <t>[18, 17, 1, 13, 8, 2, 18]</t>
+          <t>[18, 11, 13, 8, 2, 18]</t>
         </is>
       </c>
       <c r="O60" s="16" t="n">
-        <v>4424</v>
+        <v>4454</v>
       </c>
       <c r="P60" s="17" t="n">
-        <v>76.75141659465382</v>
+        <v>68.56140072641271</v>
       </c>
       <c r="Q60" s="15" t="b">
         <v>1</v>
@@ -12506,14 +12608,14 @@
       </c>
       <c r="V60" s="15" t="inlineStr">
         <is>
-          <t>[18, 11, 2, 18]</t>
+          <t>[18, 11, 13, 8, 2, 18]</t>
         </is>
       </c>
       <c r="W60" s="16" t="n">
-        <v>2370</v>
+        <v>4454</v>
       </c>
       <c r="X60" s="17" t="n">
-        <v>63.58875588680079</v>
+        <v>68.56140072641271</v>
       </c>
       <c r="Y60" s="15" t="b">
         <v>1</v>
@@ -12525,13 +12627,13 @@
         <v>1.851035698545615</v>
       </c>
       <c r="AB60" s="5" t="n">
-        <v>2.51211987659762</v>
+        <v>1.851035698545615</v>
       </c>
       <c r="AC60" s="5" t="n">
         <v>1.851035698545615</v>
       </c>
       <c r="AD60" s="5" t="n">
-        <v>47.77434993389158</v>
+        <v>1.851035698545615</v>
       </c>
       <c r="AE60" s="18" t="inlineStr">
         <is>
@@ -12582,14 +12684,14 @@
       </c>
       <c r="AR60" s="18" t="inlineStr">
         <is>
-          <t>[18, 11, 2, 18]</t>
+          <t>[18, 11, 13, 8, 2, 18]</t>
         </is>
       </c>
       <c r="AS60" s="19" t="n">
-        <v>2370</v>
+        <v>4454</v>
       </c>
       <c r="AT60" s="20" t="n">
-        <v>63.58875588680079</v>
+        <v>68.56140072641271</v>
       </c>
       <c r="AU60" s="18" t="b">
         <v>1</v>
@@ -12618,7 +12720,7 @@
         <v>1.851035698545615</v>
       </c>
       <c r="BC60" s="5" t="n">
-        <v>47.77434993389158</v>
+        <v>1.851035698545615</v>
       </c>
       <c r="BD60" s="5" t="n">
         <v>1.851035698545615</v>
@@ -13341,22 +13443,22 @@
         <v>60</v>
       </c>
       <c r="D3" t="n">
-        <v>2355.15</v>
+        <v>2404.716666666667</v>
       </c>
       <c r="E3" t="n">
-        <v>1140.613629453425</v>
+        <v>1197.181125467296</v>
       </c>
       <c r="F3" t="n">
-        <v>1734.75</v>
+        <v>1772</v>
       </c>
       <c r="G3" t="n">
-        <v>2506.5</v>
+        <v>2584.5</v>
       </c>
       <c r="H3" t="n">
-        <v>3042.25</v>
+        <v>3092.5</v>
       </c>
       <c r="I3" t="n">
-        <v>-182</v>
+        <v>-600</v>
       </c>
       <c r="J3" t="n">
         <v>6109</v>
@@ -13496,19 +13598,19 @@
         <v>60</v>
       </c>
       <c r="C2" t="n">
-        <v>1107.55</v>
+        <v>1057.983333333333</v>
       </c>
       <c r="D2" t="n">
-        <v>1020</v>
+        <v>1046</v>
       </c>
       <c r="E2" t="n">
-        <v>909.7057155932631</v>
+        <v>778.768377733837</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1.625698456933097e-10</v>
+        <v>2.386484752546066e-10</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -13573,4 +13675,416 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>CHEQUEO DE CONVERGENCIA PPO  ·  20 nodos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>CRITERIOS DE CONVERGENCIA  (evaluados sobre las últimas W = 50 PPO updates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Métrica observada</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Cómo se mide</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Umbral de aprobación</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Nota de diseño</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>C1 — Reward aplanado</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Pendiente relativa del reward de entrenamiento</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Regresión lineal sobre la ventana → slope / |media reward|</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>&lt; 0.001  (adimensional)</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Valor relativo para que sea comparable entre escalas de reward distintas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>C2 — Explained Variance estable</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Media y pendiente relativa de explained_var del crítico</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Media aritmética + regresión lineal sobre la ventana</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Media ≥ 0.5  Y  |pendiente rel.| &lt; 0.001</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Umbral 0.5 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>C3 — KL divergence controlada</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Fracción de updates en ventana con KL &gt; umbral KL</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Proporción de filas donde kl_divergence &gt; kl_threshold</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Fracción de violaciones ≤ 5%  (umbral KL = 0.02)</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Umbral KL 0.02 coincide con la línea de referencia en PPO_Diagnostics_AM.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>C4 — Entropía estabilizada</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>Pendiente ABSOLUTA de la entropía de la política</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Regresión lineal sobre la ventana → |slope| en nats/update</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>&lt; 0.0005  nats/update</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Se usa pendiente absoluta (no relativa) porque la entropía puede pasar por 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1"/>
+    <row r="10" ht="40" customHeight="1"/>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>RESULTADOS DEL CHEQUEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Identificación</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>C1 — Reward Aplanado</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="n"/>
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>C2 — Explained Variance</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="n"/>
+      <c r="I12" s="31" t="n"/>
+      <c r="J12" s="31" t="n"/>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>C3 — KL Divergence</t>
+        </is>
+      </c>
+      <c r="L12" s="32" t="n"/>
+      <c r="M12" s="32" t="n"/>
+      <c r="N12" s="33" t="inlineStr">
+        <is>
+          <t>C4 — Entropía</t>
+        </is>
+      </c>
+      <c r="O12" s="34" t="n"/>
+      <c r="P12" s="34" t="n"/>
+      <c r="Q12" s="35" t="inlineStr">
+        <is>
+          <t>Veredicto Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Nodos</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Total
+Updates</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>Ventana
+(W usado)</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Pendiente
+Reward Rel.
+(medido)</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Umbral
+(&lt; 0.001)</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>C1
+Resultado</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>EV Media
+(medido)</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>EV Pendiente
+Rel. (medido)</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Umbral
+Media ≥ 0.5</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>C2
+Resultado</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Fracc.
+Violaciones
+KL (medido)</t>
+        </is>
+      </c>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>Umbral
+(≤ 5%)</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>C3
+Resultado</t>
+        </is>
+      </c>
+      <c r="N13" s="33" t="inlineStr">
+        <is>
+          <t>Pendiente
+Entropía Abs.
+(medido)</t>
+        </is>
+      </c>
+      <c r="O13" s="33" t="inlineStr">
+        <is>
+          <t>Umbral
+(&lt; 0.0005)</t>
+        </is>
+      </c>
+      <c r="P13" s="33" t="inlineStr">
+        <is>
+          <t>C4
+Resultado</t>
+        </is>
+      </c>
+      <c r="Q13" s="35" t="inlineStr">
+        <is>
+          <t>CONVERGIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="B14" s="37" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C14" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" s="38" t="n">
+        <v>0.000185</v>
+      </c>
+      <c r="E14" s="39" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="n">
+        <v>0.8678</v>
+      </c>
+      <c r="H14" s="38" t="n">
+        <v>9.6e-05</v>
+      </c>
+      <c r="I14" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="42" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N14" s="38" t="n">
+        <v>0.000138</v>
+      </c>
+      <c r="O14" s="39" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="P14" s="40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q14" s="43" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="N12:P12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Resultados estables luego de paralelizacion nivel 2, convergencia en 20 nodos
</commit_message>
<xml_diff>
--- a/results_20nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_20nodes/DRL_Routing_Summary_AM.xlsx
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2.099132537841797</v>
+        <v>2.120554447174072</v>
       </c>
     </row>
     <row r="4">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3314.616666666667</v>
+        <v>3321.083333333333</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>6.711958732542758</v>
+        <v>6.546824241565571</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>149.0353544553121</v>
+        <v>144.1125392913818</v>
       </c>
     </row>
     <row r="5">
@@ -756,7 +756,7 @@
         <v>0.05724222139238529</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1740.631985664368</v>
+        <v>1677.107397715251</v>
       </c>
     </row>
     <row r="6">
@@ -772,7 +772,7 @@
         <v>4.612965002829824</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1.154224077860514</v>
+        <v>1.170849800109863</v>
       </c>
     </row>
     <row r="7">
@@ -788,7 +788,7 @@
         <v>39.86581939848013</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0.3040035565694173</v>
+        <v>0.2854307492574056</v>
       </c>
     </row>
     <row r="9">
@@ -836,7 +836,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>7.55076805750529</v>
+        <v>7.190100351969401</v>
       </c>
     </row>
     <row r="12">
@@ -852,7 +852,7 @@
         <v>1.940915761618184</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>149.0353544553121</v>
+        <v>144.1125392913818</v>
       </c>
     </row>
     <row r="13">
@@ -868,7 +868,7 @@
         <v>4.545012160007144</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>4.09390926361084</v>
+        <v>3.915747006734212</v>
       </c>
     </row>
     <row r="14">
@@ -898,7 +898,7 @@
         <v>7.919557852777054</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>4.095109303792318</v>
+        <v>3.939421971638998</v>
       </c>
     </row>
     <row r="17">
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>13105.90102243423</v>
+        <v>3892.783104896545</v>
       </c>
     </row>
     <row r="20">
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>149.0353544553121</v>
+        <v>144.1125392913818</v>
       </c>
     </row>
     <row r="21">
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>1740.631985664368</v>
+        <v>1677.107397715251</v>
       </c>
     </row>
     <row r="22">
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>2.099132537841797</v>
+        <v>2.120554447174072</v>
       </c>
     </row>
     <row r="23">
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.3040035565694173</v>
+        <v>0.2854307492574056</v>
       </c>
     </row>
     <row r="24">
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1.154224077860514</v>
+        <v>1.170849800109863</v>
       </c>
     </row>
     <row r="25">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>4.09390926361084</v>
+        <v>3.915747006734212</v>
       </c>
     </row>
     <row r="26">
@@ -998,7 +998,7 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>4.095109303792318</v>
+        <v>3.939421971638998</v>
       </c>
     </row>
     <row r="27">
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>7.55076805750529</v>
+        <v>7.190100351969401</v>
       </c>
     </row>
   </sheetData>
@@ -11973,14 +11973,14 @@
       </c>
       <c r="I57" s="15" t="inlineStr">
         <is>
-          <t>[17, 16, 12, 13, 17]</t>
+          <t>[17, 16, 12, 1, 13, 17]</t>
         </is>
       </c>
       <c r="J57" s="16" t="n">
-        <v>3528</v>
+        <v>3916</v>
       </c>
       <c r="K57" s="17" t="n">
-        <v>67.42434623698556</v>
+        <v>71.12444971666355</v>
       </c>
       <c r="L57" s="15" t="b">
         <v>1</v>
@@ -12036,7 +12036,7 @@
         <v>0</v>
       </c>
       <c r="AA57" s="5" t="n">
-        <v>9.908069458631257</v>
+        <v>0</v>
       </c>
       <c r="AB57" s="5" t="n">
         <v>0</v>
@@ -14016,13 +14016,13 @@
         <v>20</v>
       </c>
       <c r="B14" s="37" t="n">
-        <v>1000</v>
+        <v>833</v>
       </c>
       <c r="C14" s="37" t="n">
         <v>50</v>
       </c>
       <c r="D14" s="38" t="n">
-        <v>0.000185</v>
+        <v>0.000128</v>
       </c>
       <c r="E14" s="39" t="n">
         <v>0.001</v>
@@ -14033,10 +14033,10 @@
         </is>
       </c>
       <c r="G14" s="41" t="n">
-        <v>0.8678</v>
+        <v>0.8573</v>
       </c>
       <c r="H14" s="38" t="n">
-        <v>9.6e-05</v>
+        <v>0.000115</v>
       </c>
       <c r="I14" s="42" t="n">
         <v>0.5</v>
@@ -14058,7 +14058,7 @@
         </is>
       </c>
       <c r="N14" s="38" t="n">
-        <v>0.000138</v>
+        <v>0.000317</v>
       </c>
       <c r="O14" s="39" t="n">
         <v>0.0005</v>

</xml_diff>